<commit_message>
3.5.0: - average of 95% image (what about length < num_patches) - added return types -Histogram 3D RunTime warning
</commit_message>
<xml_diff>
--- a/results/SamChigome/Analysis_v2.xlsx
+++ b/results/SamChigome/Analysis_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/owuorjnr/Downloads/Sam Chigome/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C8BAE28-7059-FC4C-887A-BB58F943650E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB239B3-A3C5-A349-B185-7047AB53163E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9860" yWindow="2660" windowWidth="36880" windowHeight="22720" activeTab="7" xr2:uid="{E8351862-8131-4AC1-82A9-213539580791}"/>
+    <workbookView xWindow="13540" yWindow="2320" windowWidth="36880" windowHeight="22720" activeTab="7" xr2:uid="{E8351862-8131-4AC1-82A9-213539580791}"/>
   </bookViews>
   <sheets>
     <sheet name="SGT Descriptors" sheetId="2" r:id="rId1"/>
@@ -22,74 +22,6 @@
     <sheet name="Nodes-Avg. EigVec. C." sheetId="13" r:id="rId7"/>
     <sheet name="Nodes-Avg. Close. C" sheetId="14" r:id="rId8"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId9"/>
-  </externalReferences>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">'SGT Descriptors'!$B$2</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">('SGT Descriptors'!$B$3,'SGT Descriptors'!$B$4,'SGT Descriptors'!$B$5,'SGT Descriptors'!$B$7,'SGT Descriptors'!$B$8,'SGT Descriptors'!$B$9,'SGT Descriptors'!$B$10)</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">('SGT Descriptors'!$G$11,'SGT Descriptors'!$G$12,'SGT Descriptors'!$G$13,'SGT Descriptors'!$G$15,'SGT Descriptors'!$G$16,'SGT Descriptors'!$G$17,'SGT Descriptors'!$G$18)</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">('SGT Descriptors'!$G$19:$G$20,'SGT Descriptors'!$G$21,'SGT Descriptors'!$G$23,'SGT Descriptors'!$G$24,'SGT Descriptors'!$G$25,'SGT Descriptors'!$G$26)</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">('SGT Descriptors'!$G$27,'SGT Descriptors'!$G$28,'SGT Descriptors'!$G$29,'SGT Descriptors'!$G$31,'SGT Descriptors'!$G$32,'SGT Descriptors'!$G$33,'SGT Descriptors'!$G$34)</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">('SGT Descriptors'!$G$3,'SGT Descriptors'!$G$4,'SGT Descriptors'!$G$5,'SGT Descriptors'!$G$7,'SGT Descriptors'!$G$8,'SGT Descriptors'!$G$9,'SGT Descriptors'!$G$10)</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">'SGT Descriptors'!$B$2</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">('SGT Descriptors'!$B$3,'SGT Descriptors'!$B$4,'SGT Descriptors'!$B$5,'SGT Descriptors'!$B$7,'SGT Descriptors'!$B$8,'SGT Descriptors'!$B$9,'SGT Descriptors'!$B$10)</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">('SGT Descriptors'!$G$11,'SGT Descriptors'!$G$12,'SGT Descriptors'!$G$13,'SGT Descriptors'!$G$15,'SGT Descriptors'!$G$16,'SGT Descriptors'!$G$17,'SGT Descriptors'!$G$18)</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">('SGT Descriptors'!$G$19:$G$20,'SGT Descriptors'!$G$21,'SGT Descriptors'!$G$23,'SGT Descriptors'!$G$24,'SGT Descriptors'!$G$25,'SGT Descriptors'!$G$26)</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">('SGT Descriptors'!$G$27,'SGT Descriptors'!$G$28,'SGT Descriptors'!$G$29,'SGT Descriptors'!$G$31,'SGT Descriptors'!$G$32,'SGT Descriptors'!$G$33,'SGT Descriptors'!$G$34)</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">('SGT Descriptors'!$G$3,'SGT Descriptors'!$G$4,'SGT Descriptors'!$G$5,'SGT Descriptors'!$G$7,'SGT Descriptors'!$G$8,'SGT Descriptors'!$G$9,'SGT Descriptors'!$G$10)</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'SGT Descriptors'!$B$2</definedName>
-    <definedName name="_xlchart.v1.30" hidden="1">'SGT Descriptors'!$B$2</definedName>
-    <definedName name="_xlchart.v1.31" hidden="1">('SGT Descriptors'!$B$3,'SGT Descriptors'!$B$4,'SGT Descriptors'!$B$5,'SGT Descriptors'!$B$7,'SGT Descriptors'!$B$8,'SGT Descriptors'!$B$9,'SGT Descriptors'!$B$10)</definedName>
-    <definedName name="_xlchart.v1.32" hidden="1">('SGT Descriptors'!$G$11,'SGT Descriptors'!$G$12,'SGT Descriptors'!$G$13,'SGT Descriptors'!$G$15,'SGT Descriptors'!$G$16,'SGT Descriptors'!$G$17,'SGT Descriptors'!$G$18)</definedName>
-    <definedName name="_xlchart.v1.33" hidden="1">('SGT Descriptors'!$G$19:$G$20,'SGT Descriptors'!$G$21,'SGT Descriptors'!$G$23,'SGT Descriptors'!$G$24,'SGT Descriptors'!$G$25,'SGT Descriptors'!$G$26)</definedName>
-    <definedName name="_xlchart.v1.34" hidden="1">('SGT Descriptors'!$G$27,'SGT Descriptors'!$G$28,'SGT Descriptors'!$G$29,'SGT Descriptors'!$G$31,'SGT Descriptors'!$G$32,'SGT Descriptors'!$G$33,'SGT Descriptors'!$G$34)</definedName>
-    <definedName name="_xlchart.v1.35" hidden="1">('SGT Descriptors'!$G$3,'SGT Descriptors'!$G$4,'SGT Descriptors'!$G$5,'SGT Descriptors'!$G$7,'SGT Descriptors'!$G$8,'SGT Descriptors'!$G$9,'SGT Descriptors'!$G$10)</definedName>
-    <definedName name="_xlchart.v1.36" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.37" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.38" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.39" hidden="1">'SGT Descriptors'!$B$2</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">('SGT Descriptors'!$B$3,'SGT Descriptors'!$B$4,'SGT Descriptors'!$B$5,'SGT Descriptors'!$B$7,'SGT Descriptors'!$B$8,'SGT Descriptors'!$B$9,'SGT Descriptors'!$B$10)</definedName>
-    <definedName name="_xlchart.v1.40" hidden="1">('SGT Descriptors'!$B$3,'SGT Descriptors'!$B$4,'SGT Descriptors'!$B$5,'SGT Descriptors'!$B$7,'SGT Descriptors'!$B$8,'SGT Descriptors'!$B$9,'SGT Descriptors'!$B$10)</definedName>
-    <definedName name="_xlchart.v1.41" hidden="1">('SGT Descriptors'!$G$11,'SGT Descriptors'!$G$12,'SGT Descriptors'!$G$13,'SGT Descriptors'!$G$15,'SGT Descriptors'!$G$16,'SGT Descriptors'!$G$17,'SGT Descriptors'!$G$18)</definedName>
-    <definedName name="_xlchart.v1.42" hidden="1">('SGT Descriptors'!$G$19:$G$20,'SGT Descriptors'!$G$21,'SGT Descriptors'!$G$23,'SGT Descriptors'!$G$24,'SGT Descriptors'!$G$25,'SGT Descriptors'!$G$26)</definedName>
-    <definedName name="_xlchart.v1.43" hidden="1">('SGT Descriptors'!$G$27,'SGT Descriptors'!$G$28,'SGT Descriptors'!$G$29,'SGT Descriptors'!$G$31,'SGT Descriptors'!$G$32,'SGT Descriptors'!$G$33,'SGT Descriptors'!$G$34)</definedName>
-    <definedName name="_xlchart.v1.44" hidden="1">('SGT Descriptors'!$G$3,'SGT Descriptors'!$G$4,'SGT Descriptors'!$G$5,'SGT Descriptors'!$G$7,'SGT Descriptors'!$G$8,'SGT Descriptors'!$G$9,'SGT Descriptors'!$G$10)</definedName>
-    <definedName name="_xlchart.v1.45" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.46" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.47" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.48" hidden="1">'SGT Descriptors'!$B$2</definedName>
-    <definedName name="_xlchart.v1.49" hidden="1">('SGT Descriptors'!$B$3,'SGT Descriptors'!$B$4,'SGT Descriptors'!$B$5,'SGT Descriptors'!$B$7,'SGT Descriptors'!$B$8,'SGT Descriptors'!$B$9,'SGT Descriptors'!$B$10)</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">('SGT Descriptors'!$G$11,'SGT Descriptors'!$G$12,'SGT Descriptors'!$G$13,'SGT Descriptors'!$G$15,'SGT Descriptors'!$G$16,'SGT Descriptors'!$G$17,'SGT Descriptors'!$G$18)</definedName>
-    <definedName name="_xlchart.v1.50" hidden="1">('SGT Descriptors'!$G$11,'SGT Descriptors'!$G$12,'SGT Descriptors'!$G$13,'SGT Descriptors'!$G$15,'SGT Descriptors'!$G$16,'SGT Descriptors'!$G$17,'SGT Descriptors'!$G$18)</definedName>
-    <definedName name="_xlchart.v1.51" hidden="1">('SGT Descriptors'!$G$19:$G$20,'SGT Descriptors'!$G$21,'SGT Descriptors'!$G$23,'SGT Descriptors'!$G$24,'SGT Descriptors'!$G$25,'SGT Descriptors'!$G$26)</definedName>
-    <definedName name="_xlchart.v1.52" hidden="1">('SGT Descriptors'!$G$27,'SGT Descriptors'!$G$28,'SGT Descriptors'!$G$29,'SGT Descriptors'!$G$31,'SGT Descriptors'!$G$32,'SGT Descriptors'!$G$33,'SGT Descriptors'!$G$34)</definedName>
-    <definedName name="_xlchart.v1.53" hidden="1">('SGT Descriptors'!$G$3,'SGT Descriptors'!$G$4,'SGT Descriptors'!$G$5,'SGT Descriptors'!$G$7,'SGT Descriptors'!$G$8,'SGT Descriptors'!$G$9,'SGT Descriptors'!$G$10)</definedName>
-    <definedName name="_xlchart.v1.54" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.55" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.56" hidden="1">'SGT Descriptors'!#REF!</definedName>
-    <definedName name="_xlchart.v1.57" hidden="1">'SGT Descriptors'!$B$2</definedName>
-    <definedName name="_xlchart.v1.58" hidden="1">('SGT Descriptors'!$B$3,'SGT Descriptors'!$B$4,'SGT Descriptors'!$B$5,'SGT Descriptors'!$B$7,'SGT Descriptors'!$B$8,'SGT Descriptors'!$B$9,'SGT Descriptors'!$B$10)</definedName>
-    <definedName name="_xlchart.v1.59" hidden="1">('SGT Descriptors'!$G$11,'SGT Descriptors'!$G$12,'SGT Descriptors'!$G$13,'SGT Descriptors'!$G$15,'SGT Descriptors'!$G$16,'SGT Descriptors'!$G$17,'SGT Descriptors'!$G$18)</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">('SGT Descriptors'!$G$19:$G$20,'SGT Descriptors'!$G$21,'SGT Descriptors'!$G$23,'SGT Descriptors'!$G$24,'SGT Descriptors'!$G$25,'SGT Descriptors'!$G$26)</definedName>
-    <definedName name="_xlchart.v1.60" hidden="1">('SGT Descriptors'!$G$19:$G$20,'SGT Descriptors'!$G$21,'SGT Descriptors'!$G$23,'SGT Descriptors'!$G$24,'SGT Descriptors'!$G$25,'SGT Descriptors'!$G$26)</definedName>
-    <definedName name="_xlchart.v1.61" hidden="1">('SGT Descriptors'!$G$27,'SGT Descriptors'!$G$28,'SGT Descriptors'!$G$29,'SGT Descriptors'!$G$31,'SGT Descriptors'!$G$32,'SGT Descriptors'!$G$33,'SGT Descriptors'!$G$34)</definedName>
-    <definedName name="_xlchart.v1.62" hidden="1">('SGT Descriptors'!$G$3,'SGT Descriptors'!$G$4,'SGT Descriptors'!$G$5,'SGT Descriptors'!$G$7,'SGT Descriptors'!$G$8,'SGT Descriptors'!$G$9,'SGT Descriptors'!$G$10)</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">('SGT Descriptors'!$G$27,'SGT Descriptors'!$G$28,'SGT Descriptors'!$G$29,'SGT Descriptors'!$G$31,'SGT Descriptors'!$G$32,'SGT Descriptors'!$G$33,'SGT Descriptors'!$G$34)</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">('SGT Descriptors'!$G$3,'SGT Descriptors'!$G$4,'SGT Descriptors'!$G$5,'SGT Descriptors'!$G$7,'SGT Descriptors'!$G$8,'SGT Descriptors'!$G$9,'SGT Descriptors'!$G$10)</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">'SGT Descriptors'!#REF!</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -111,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="34">
   <si>
     <t>ND</t>
   </si>
@@ -523,7 +455,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4886,186 +4818,6 @@
 </c:userShapes>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Sample 3"/>
-      <sheetName val="Sample 4"/>
-      <sheetName val="Sample 5"/>
-      <sheetName val="Sample 6"/>
-      <sheetName val="All Samples"/>
-      <sheetName val="Scaling Laws"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4">
-        <row r="21">
-          <cell r="C21" t="str">
-            <v>ND</v>
-          </cell>
-          <cell r="D21" t="str">
-            <v>CC</v>
-          </cell>
-          <cell r="E21" t="str">
-            <v>BC</v>
-          </cell>
-          <cell r="F21" t="str">
-            <v>AC</v>
-          </cell>
-          <cell r="G21" t="str">
-            <v>GD</v>
-          </cell>
-          <cell r="H21" t="str">
-            <v>Nodes</v>
-          </cell>
-          <cell r="I21" t="str">
-            <v>Edges</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="B22" t="str">
-            <v>BSE 010</v>
-          </cell>
-          <cell r="C22">
-            <v>4.069</v>
-          </cell>
-          <cell r="D22">
-            <v>0.248</v>
-          </cell>
-          <cell r="E22">
-            <v>4.0000000000000001E-3</v>
-          </cell>
-          <cell r="F22">
-            <v>-0.122</v>
-          </cell>
-          <cell r="G22">
-            <v>5.0000000000000001E-4</v>
-          </cell>
-          <cell r="H22">
-            <v>8093</v>
-          </cell>
-          <cell r="I22">
-            <v>16466</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="B23" t="str">
-            <v>BSE 011</v>
-          </cell>
-          <cell r="C23">
-            <v>4.0350000000000001</v>
-          </cell>
-          <cell r="D23">
-            <v>0.24</v>
-          </cell>
-          <cell r="E23">
-            <v>4.0000000000000001E-3</v>
-          </cell>
-          <cell r="F23">
-            <v>-0.128</v>
-          </cell>
-          <cell r="G23">
-            <v>5.0000000000000001E-4</v>
-          </cell>
-          <cell r="H23">
-            <v>8248</v>
-          </cell>
-          <cell r="I23">
-            <v>16639</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="B24" t="str">
-            <v>BSE 017</v>
-          </cell>
-          <cell r="C24">
-            <v>3.8849999999999998</v>
-          </cell>
-          <cell r="D24">
-            <v>0.20899999999999999</v>
-          </cell>
-          <cell r="E24">
-            <v>4.0000000000000001E-3</v>
-          </cell>
-          <cell r="F24">
-            <v>-0.111</v>
-          </cell>
-          <cell r="G24">
-            <v>4.0000000000000002E-4</v>
-          </cell>
-          <cell r="H24">
-            <v>9080</v>
-          </cell>
-          <cell r="I24">
-            <v>17638</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="B25" t="str">
-            <v>BSE 024</v>
-          </cell>
-          <cell r="C25">
-            <v>3.9350000000000001</v>
-          </cell>
-          <cell r="D25">
-            <v>0.221</v>
-          </cell>
-          <cell r="E25">
-            <v>4.0000000000000001E-3</v>
-          </cell>
-          <cell r="F25">
-            <v>-0.1056</v>
-          </cell>
-          <cell r="G25">
-            <v>4.0000000000000002E-4</v>
-          </cell>
-          <cell r="H25">
-            <v>8840</v>
-          </cell>
-          <cell r="I25">
-            <v>17393</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="B26" t="str">
-            <v>BSE 025</v>
-          </cell>
-          <cell r="C26">
-            <v>3.8159999999999998</v>
-          </cell>
-          <cell r="D26">
-            <v>0.21</v>
-          </cell>
-          <cell r="E26">
-            <v>4.0000000000000001E-3</v>
-          </cell>
-          <cell r="F26">
-            <v>-0.11799999999999999</v>
-          </cell>
-          <cell r="G26">
-            <v>5.0000000000000001E-4</v>
-          </cell>
-          <cell r="H26">
-            <v>8566</v>
-          </cell>
-          <cell r="I26">
-            <v>16344</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="5" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -6361,6 +6113,9 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>25</v>
+      </c>
       <c r="B2" s="26" t="s">
         <v>26</v>
       </c>
@@ -7680,6 +7435,9 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>25</v>
+      </c>
       <c r="B2" s="28" t="s">
         <v>26</v>
       </c>
@@ -9009,7 +8767,9 @@
       <c r="I1" s="27"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="27"/>
+      <c r="A2" s="21" t="s">
+        <v>25</v>
+      </c>
       <c r="B2" s="28" t="s">
         <v>26</v>
       </c>
@@ -10342,7 +10102,9 @@
       <c r="I1" s="27"/>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A2" s="27"/>
+      <c r="A2" s="21" t="s">
+        <v>25</v>
+      </c>
       <c r="B2" s="28" t="s">
         <v>26</v>
       </c>
@@ -11623,7 +11385,7 @@
       <c r="E44" s="22">
         <v>3.6700999999999998E-2</v>
       </c>
-      <c r="F44" s="31">
+      <c r="F44" s="22">
         <v>4.6100000000000002E-5</v>
       </c>
       <c r="G44" s="22">
@@ -11652,7 +11414,7 @@
       <c r="E45" s="22">
         <v>3.3259999999999998E-2</v>
       </c>
-      <c r="F45" s="31">
+      <c r="F45" s="22">
         <v>2.0299999999999999E-5</v>
       </c>
       <c r="G45" s="22">
@@ -11703,21 +11465,22 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{908D8F90-1399-4559-8642-02E0AC650D8E}">
-  <dimension ref="B1:AD46"/>
+  <dimension ref="A1:AC46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.6640625" customWidth="1"/>
-    <col min="3" max="3" width="10.1640625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" style="6" customWidth="1"/>
-    <col min="5" max="6" width="10.5" style="6" customWidth="1"/>
-    <col min="7" max="14" width="9.5" style="7" customWidth="1"/>
-    <col min="15" max="18" width="9.1640625" style="8"/>
-    <col min="19" max="22" width="9.1640625" style="9"/>
-    <col min="23" max="26" width="9.5" style="7" customWidth="1"/>
-    <col min="27" max="30" width="9.1640625" style="10"/>
+    <col min="1" max="1" width="11.6640625" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" style="6" customWidth="1"/>
+    <col min="4" max="5" width="10.5" style="6" customWidth="1"/>
+    <col min="6" max="13" width="9.5" style="7" customWidth="1"/>
+    <col min="14" max="17" width="9.1640625" style="8"/>
+    <col min="18" max="21" width="9.1640625" style="9"/>
+    <col min="22" max="25" width="9.5" style="7" customWidth="1"/>
+    <col min="26" max="29" width="9.1640625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:30" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A1" s="27"/>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
       <c r="D1" s="27"/>
@@ -11726,1388 +11489,1389 @@
       <c r="G1" s="27"/>
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-    </row>
-    <row r="2" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B2" s="27"/>
-      <c r="C2" s="28" t="s">
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="28" t="s">
         <v>26</v>
       </c>
+      <c r="C2" s="29" t="s">
+        <v>27</v>
+      </c>
       <c r="D2" s="29" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E2" s="29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" s="29" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G2" s="29" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H2" s="29" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I2" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="J2" s="29" t="s">
         <v>33</v>
       </c>
+      <c r="J2" s="14"/>
       <c r="K2" s="14"/>
       <c r="L2" s="14"/>
       <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
+      <c r="V2" s="16"/>
       <c r="W2" s="16"/>
       <c r="X2" s="16"/>
       <c r="Y2" s="16"/>
-      <c r="Z2" s="16"/>
-    </row>
-    <row r="3" spans="2:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="27" t="s">
+    </row>
+    <row r="3" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
       <c r="C3">
-        <v>65</v>
+        <v>54.1</v>
       </c>
       <c r="D3">
-        <v>54.1</v>
+        <v>2.1105554824368968</v>
       </c>
       <c r="E3">
-        <v>2.1105554824368968</v>
+        <v>0.21757000000000001</v>
       </c>
       <c r="F3">
-        <v>0.21757000000000001</v>
+        <v>4.4148104275394569E-3</v>
       </c>
       <c r="G3">
-        <v>4.4148104275394569E-3</v>
+        <v>1.733197265106569</v>
       </c>
       <c r="H3">
-        <v>1.733197265106569</v>
+        <v>-0.66240098826001137</v>
       </c>
       <c r="I3">
-        <v>-0.66240098826001137</v>
-      </c>
-      <c r="J3">
         <v>-0.6483143837514157</v>
       </c>
+      <c r="J3" s="15"/>
       <c r="K3" s="15"/>
       <c r="L3" s="15"/>
       <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
+      <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+      <c r="R3" s="18"/>
       <c r="S3" s="18"/>
       <c r="T3" s="18"/>
       <c r="U3" s="18"/>
-      <c r="V3" s="18"/>
+      <c r="V3" s="17"/>
       <c r="W3" s="17"/>
       <c r="X3" s="17"/>
       <c r="Y3" s="17"/>
-      <c r="Z3" s="17"/>
+      <c r="Z3" s="13"/>
       <c r="AA3" s="13"/>
       <c r="AB3" s="13"/>
       <c r="AC3" s="13"/>
-      <c r="AD3" s="13"/>
-    </row>
-    <row r="4" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B4" s="27" t="s">
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A4" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B4">
+        <v>131</v>
+      </c>
       <c r="C4">
-        <v>131</v>
+        <v>216.5</v>
       </c>
       <c r="D4">
-        <v>216.5</v>
+        <v>2.486630920207769</v>
       </c>
       <c r="E4">
-        <v>2.486630920207769</v>
+        <v>0.122269</v>
       </c>
       <c r="F4">
-        <v>0.122269</v>
+        <v>1.696034885647501E-3</v>
       </c>
       <c r="G4">
-        <v>1.696034885647501E-3</v>
+        <v>2.3354579006893839</v>
       </c>
       <c r="H4">
-        <v>2.3354579006893839</v>
+        <v>-0.91268363973813083</v>
       </c>
       <c r="I4">
-        <v>-0.91268363973813083</v>
-      </c>
-      <c r="J4">
         <v>-0.9100379661162683</v>
       </c>
+      <c r="J4" s="14"/>
       <c r="K4" s="14"/>
       <c r="L4" s="14"/>
       <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
+      <c r="V4" s="16"/>
       <c r="W4" s="16"/>
       <c r="X4" s="16"/>
       <c r="Y4" s="16"/>
-      <c r="Z4" s="16"/>
-    </row>
-    <row r="5" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B5" s="27" t="s">
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>196</v>
+      </c>
       <c r="C5">
-        <v>196</v>
+        <v>475.2</v>
       </c>
       <c r="D5">
-        <v>475.2</v>
+        <v>4.6804558182581601</v>
       </c>
       <c r="E5">
-        <v>4.6804558182581601</v>
+        <v>8.8970999999999995E-2</v>
       </c>
       <c r="F5">
-        <v>8.8970999999999995E-2</v>
+        <v>1.258028837330669E-3</v>
       </c>
       <c r="G5">
-        <v>1.258028837330669E-3</v>
+        <v>2.6768764319731368</v>
       </c>
       <c r="H5">
-        <v>2.6768764319731368</v>
+        <v>-1.050751528100486</v>
       </c>
       <c r="I5">
-        <v>-1.050751528100486</v>
-      </c>
-      <c r="J5">
         <v>-1.0584077512456891</v>
       </c>
+      <c r="J5" s="14"/>
       <c r="K5" s="14"/>
       <c r="L5" s="14"/>
       <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
+      <c r="V5" s="16"/>
       <c r="W5" s="16"/>
       <c r="X5" s="16"/>
       <c r="Y5" s="16"/>
-      <c r="Z5" s="16"/>
-    </row>
-    <row r="6" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B6" s="27" t="s">
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A6" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>262</v>
+      </c>
       <c r="C6">
-        <v>262</v>
+        <v>867.1</v>
       </c>
       <c r="D6">
-        <v>867.1</v>
+        <v>5.5486735151545714</v>
       </c>
       <c r="E6">
-        <v>5.5486735151545714</v>
+        <v>6.9492999999999999E-2</v>
       </c>
       <c r="F6">
-        <v>6.9492999999999999E-2</v>
+        <v>7.1478831365190431E-4</v>
       </c>
       <c r="G6">
-        <v>7.1478831365190431E-4</v>
+        <v>2.9380691862233861</v>
       </c>
       <c r="H6">
-        <v>2.9380691862233861</v>
+        <v>-1.1580589395031271</v>
       </c>
       <c r="I6">
-        <v>-1.1580589395031271</v>
-      </c>
-      <c r="J6">
         <v>-1.1719139299517971</v>
       </c>
+      <c r="J6" s="14"/>
       <c r="K6" s="14"/>
       <c r="L6" s="14"/>
       <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
+      <c r="V6" s="16"/>
       <c r="W6" s="16"/>
       <c r="X6" s="16"/>
       <c r="Y6" s="16"/>
-      <c r="Z6" s="16"/>
-    </row>
-    <row r="7" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B7" s="27" t="s">
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A7" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B7">
+        <v>328</v>
+      </c>
       <c r="C7">
-        <v>328</v>
+        <v>1347.8</v>
       </c>
       <c r="D7">
-        <v>1347.8</v>
+        <v>9.7431457388714495</v>
       </c>
       <c r="E7">
-        <v>9.7431457388714495</v>
+        <v>5.6467999999999997E-2</v>
       </c>
       <c r="F7">
-        <v>5.6467999999999997E-2</v>
+        <v>3.919688196216065E-4</v>
       </c>
       <c r="G7">
-        <v>3.919688196216065E-4</v>
+        <v>3.129625452035683</v>
       </c>
       <c r="H7">
-        <v>3.129625452035683</v>
+        <v>-1.2481975939586329</v>
       </c>
       <c r="I7">
-        <v>-1.2481975939586329</v>
-      </c>
-      <c r="J7">
         <v>-1.255158274925984</v>
       </c>
+      <c r="J7" s="14"/>
       <c r="K7" s="14"/>
       <c r="L7" s="14"/>
       <c r="M7" s="14"/>
-      <c r="N7" s="14"/>
+      <c r="V7" s="16"/>
       <c r="W7" s="16"/>
       <c r="X7" s="16"/>
       <c r="Y7" s="16"/>
-      <c r="Z7" s="16"/>
-    </row>
-    <row r="8" spans="2:30" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="27" t="s">
+    </row>
+    <row r="8" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B8">
+        <v>393</v>
+      </c>
       <c r="C8">
-        <v>393</v>
+        <v>1958</v>
       </c>
       <c r="D8">
-        <v>1958</v>
+        <v>6.7214416443035319</v>
       </c>
       <c r="E8">
-        <v>6.7214416443035319</v>
+        <v>4.8088000000000013E-2</v>
       </c>
       <c r="F8">
-        <v>4.8088000000000013E-2</v>
+        <v>1.7630655121123509E-4</v>
       </c>
       <c r="G8">
-        <v>1.7630655121123509E-4</v>
+        <v>3.291812687467119</v>
       </c>
       <c r="H8">
-        <v>3.291812687467119</v>
+        <v>-1.31796328503944</v>
       </c>
       <c r="I8">
-        <v>-1.31796328503944</v>
-      </c>
-      <c r="J8">
         <v>-1.3256397604540711</v>
       </c>
+      <c r="J8" s="15"/>
       <c r="K8" s="15"/>
       <c r="L8" s="15"/>
       <c r="M8" s="15"/>
-      <c r="N8" s="15"/>
+      <c r="N8" s="11"/>
       <c r="O8" s="11"/>
       <c r="P8" s="11"/>
       <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
+      <c r="R8" s="12"/>
       <c r="S8" s="12"/>
       <c r="T8" s="12"/>
       <c r="U8" s="12"/>
-      <c r="V8" s="12"/>
+      <c r="V8" s="17"/>
       <c r="W8" s="17"/>
       <c r="X8" s="17"/>
       <c r="Y8" s="17"/>
-      <c r="Z8" s="17"/>
+      <c r="Z8" s="13"/>
       <c r="AA8" s="13"/>
       <c r="AB8" s="13"/>
       <c r="AC8" s="13"/>
-      <c r="AD8" s="13"/>
-    </row>
-    <row r="9" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B9" s="27" t="s">
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A9" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B9">
+        <v>459</v>
+      </c>
       <c r="C9">
-        <v>459</v>
+        <v>2654.7</v>
       </c>
       <c r="D9">
-        <v>2654.7</v>
+        <v>7.4893257373411126</v>
       </c>
       <c r="E9">
-        <v>7.4893257373411126</v>
+        <v>4.1514000000000002E-2</v>
       </c>
       <c r="F9">
-        <v>4.1514000000000002E-2</v>
+        <v>1.0577964517492631E-4</v>
       </c>
       <c r="G9">
-        <v>1.0577964517492631E-4</v>
+        <v>3.4240154498219888</v>
       </c>
       <c r="H9">
-        <v>3.4240154498219888</v>
+        <v>-1.3818054190128619</v>
       </c>
       <c r="I9">
-        <v>-1.3818054190128619</v>
-      </c>
-      <c r="J9">
         <v>-1.383090934443822</v>
       </c>
     </row>
-    <row r="10" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B10" s="27" t="s">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A10" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B10">
+        <v>524</v>
+      </c>
       <c r="C10">
+        <v>3471.9</v>
+      </c>
+      <c r="D10">
+        <v>7.8760537213900612</v>
+      </c>
+      <c r="E10">
+        <v>3.7012999999999997E-2</v>
+      </c>
+      <c r="F10">
+        <v>7.2817122528518924E-5</v>
+      </c>
+      <c r="G10">
+        <v>3.5405672078426962</v>
+      </c>
+      <c r="H10">
+        <v>-1.43164571277997</v>
+      </c>
+      <c r="I10">
+        <v>-1.4337406728425159</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A11" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11">
+        <v>590</v>
+      </c>
+      <c r="C11">
+        <v>4413.5</v>
+      </c>
+      <c r="D11">
+        <v>4.8125992053266922</v>
+      </c>
+      <c r="E11">
+        <v>3.3245999999999998E-2</v>
+      </c>
+      <c r="F11">
+        <v>4.7215816559001928E-5</v>
+      </c>
+      <c r="G11">
+        <v>3.6447831309233569</v>
+      </c>
+      <c r="H11">
+        <v>-1.4782605994564519</v>
+      </c>
+      <c r="I11">
+        <v>-1.4790296442887989</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A12" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12">
+        <v>656</v>
+      </c>
+      <c r="C12">
+        <v>5462.5</v>
+      </c>
+      <c r="D12">
+        <v>5.2983225857078793</v>
+      </c>
+      <c r="E12">
+        <v>3.0091E-2</v>
+      </c>
+      <c r="F12">
+        <v>1.7285189549952141E-5</v>
+      </c>
+      <c r="G12">
+        <v>3.7373914499784782</v>
+      </c>
+      <c r="H12">
+        <v>-1.521563379316567</v>
+      </c>
+      <c r="I12">
+        <v>-1.5192743150972079</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A13" s="27" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13">
+        <v>666</v>
+      </c>
+      <c r="C13">
+        <v>8615</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>2.3630000000000009E-2</v>
+      </c>
+      <c r="F13">
+        <v>1.1564823173178709E-18</v>
+      </c>
+      <c r="G13">
+        <v>3.9352552817840469</v>
+      </c>
+      <c r="H13">
+        <v>-1.6265362783676309</v>
+      </c>
+      <c r="I13">
+        <v>-1.6052597304157381</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A14" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14">
+        <v>65</v>
+      </c>
+      <c r="C14">
+        <v>47.8</v>
+      </c>
+      <c r="D14">
+        <v>1.481740718059525</v>
+      </c>
+      <c r="E14">
+        <v>0.20963699999999999</v>
+      </c>
+      <c r="F14">
+        <v>8.4001738143392648E-3</v>
+      </c>
+      <c r="G14">
+        <v>1.679427896612119</v>
+      </c>
+      <c r="H14">
+        <v>-0.67853206387484444</v>
+      </c>
+      <c r="I14">
+        <v>-0.65745448535624873</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A15" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15">
+        <v>130</v>
+      </c>
+      <c r="C15">
+        <v>201.9</v>
+      </c>
+      <c r="D15">
+        <v>3.813572253587616</v>
+      </c>
+      <c r="E15">
+        <v>0.12109300000000001</v>
+      </c>
+      <c r="F15">
+        <v>3.5074850280824039E-3</v>
+      </c>
+      <c r="G15">
+        <v>2.3051363189436391</v>
+      </c>
+      <c r="H15">
+        <v>-0.91688096130979457</v>
+      </c>
+      <c r="I15">
+        <v>-0.93221109867613228</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A16" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>196</v>
+      </c>
+      <c r="C16">
+        <v>453</v>
+      </c>
+      <c r="D16">
+        <v>4.7539457296018854</v>
+      </c>
+      <c r="E16">
+        <v>8.2914000000000015E-2</v>
+      </c>
+      <c r="F16">
+        <v>1.122124176135005E-3</v>
+      </c>
+      <c r="G16">
+        <v>2.6560982020128319</v>
+      </c>
+      <c r="H16">
+        <v>-1.0813721327862229</v>
+      </c>
+      <c r="I16">
+        <v>-1.086322974039972</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A17" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17">
+        <v>262</v>
+      </c>
+      <c r="C17">
+        <v>828.6</v>
+      </c>
+      <c r="D17">
+        <v>7.001904502823975</v>
+      </c>
+      <c r="E17">
+        <v>6.3450999999999994E-2</v>
+      </c>
+      <c r="F17">
+        <v>5.8089863334511436E-4</v>
+      </c>
+      <c r="G17">
+        <v>2.9183449289622749</v>
+      </c>
+      <c r="H17">
+        <v>-1.1975615289505279</v>
+      </c>
+      <c r="I17">
+        <v>-1.201478883692531</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A18" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18">
+        <v>327</v>
+      </c>
+      <c r="C18">
+        <v>1287.8</v>
+      </c>
+      <c r="D18">
+        <v>4.2551929059287863</v>
+      </c>
+      <c r="E18">
+        <v>5.297799999999999E-2</v>
+      </c>
+      <c r="F18">
+        <v>4.0885694319651712E-4</v>
+      </c>
+      <c r="G18">
+        <v>3.109848420756105</v>
+      </c>
+      <c r="H18">
+        <v>-1.2759044410059239</v>
+      </c>
+      <c r="I18">
+        <v>-1.285570529203939</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A19" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19">
+        <v>393</v>
+      </c>
+      <c r="C19">
+        <v>1847</v>
+      </c>
+      <c r="D19">
+        <v>6.2307481270086829</v>
+      </c>
+      <c r="E19">
+        <v>4.4794E-2</v>
+      </c>
+      <c r="F19">
+        <v>2.9242358925975057E-4</v>
+      </c>
+      <c r="G19">
+        <v>3.2664668954402409</v>
+      </c>
+      <c r="H19">
+        <v>-1.3487801543366851</v>
+      </c>
+      <c r="I19">
+        <v>-1.3543437151668081</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A20" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20">
+        <v>458</v>
+      </c>
+      <c r="C20">
+        <v>2522.6999999999998</v>
+      </c>
+      <c r="D20">
+        <v>6.4412731660751668</v>
+      </c>
+      <c r="E20">
+        <v>3.8827E-2</v>
+      </c>
+      <c r="F20">
+        <v>1.6180269191552729E-4</v>
+      </c>
+      <c r="G20">
+        <v>3.401865607199611</v>
+      </c>
+      <c r="H20">
+        <v>-1.4108661642769911</v>
+      </c>
+      <c r="I20">
+        <v>-1.413799030395358</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A21" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21">
         <v>524</v>
       </c>
-      <c r="D10">
-        <v>3471.9</v>
-      </c>
-      <c r="E10">
-        <v>7.8760537213900612</v>
-      </c>
-      <c r="F10">
-        <v>3.7012999999999997E-2</v>
-      </c>
-      <c r="G10">
-        <v>7.2817122528518924E-5</v>
-      </c>
-      <c r="H10">
-        <v>3.5405672078426962</v>
-      </c>
-      <c r="I10">
-        <v>-1.43164571277997</v>
-      </c>
-      <c r="J10">
-        <v>-1.4337406728425159</v>
-      </c>
-    </row>
-    <row r="11" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B11" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11">
-        <v>590</v>
-      </c>
-      <c r="D11">
-        <v>4413.5</v>
-      </c>
-      <c r="E11">
-        <v>4.8125992053266922</v>
-      </c>
-      <c r="F11">
-        <v>3.3245999999999998E-2</v>
-      </c>
-      <c r="G11">
-        <v>4.7215816559001928E-5</v>
-      </c>
-      <c r="H11">
-        <v>3.6447831309233569</v>
-      </c>
-      <c r="I11">
-        <v>-1.4782605994564519</v>
-      </c>
-      <c r="J11">
-        <v>-1.4790296442887989</v>
-      </c>
-    </row>
-    <row r="12" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B12" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12">
-        <v>656</v>
-      </c>
-      <c r="D12">
-        <v>5462.5</v>
-      </c>
-      <c r="E12">
-        <v>5.2983225857078793</v>
-      </c>
-      <c r="F12">
-        <v>3.0091E-2</v>
-      </c>
-      <c r="G12">
-        <v>1.7285189549952141E-5</v>
-      </c>
-      <c r="H12">
-        <v>3.7373914499784782</v>
-      </c>
-      <c r="I12">
-        <v>-1.521563379316567</v>
-      </c>
-      <c r="J12">
-        <v>-1.5192743150972079</v>
-      </c>
-    </row>
-    <row r="13" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B13" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13">
-        <v>666</v>
-      </c>
-      <c r="D13">
-        <v>8615</v>
-      </c>
-      <c r="E13">
+      <c r="C21">
+        <v>3294.9</v>
+      </c>
+      <c r="D21">
+        <v>4.3879886559156516</v>
+      </c>
+      <c r="E21">
+        <v>3.4486999999999997E-2</v>
+      </c>
+      <c r="F21">
+        <v>1.064273356698253E-4</v>
+      </c>
+      <c r="G21">
+        <v>3.5178422383208559</v>
+      </c>
+      <c r="H21">
+        <v>-1.4623445829626329</v>
+      </c>
+      <c r="I21">
+        <v>-1.4647258602954349</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A22" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B22">
+        <v>589</v>
+      </c>
+      <c r="C22">
+        <v>4152.6000000000004</v>
+      </c>
+      <c r="D22">
+        <v>5.2877216265609137</v>
+      </c>
+      <c r="E22">
+        <v>3.0827E-2</v>
+      </c>
+      <c r="F22">
+        <v>7.7374270773803059E-5</v>
+      </c>
+      <c r="G22">
+        <v>3.6183200996244</v>
+      </c>
+      <c r="H22">
+        <v>-1.511068737577747</v>
+      </c>
+      <c r="I22">
+        <v>-1.508846981092431</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A23" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23">
+        <v>655</v>
+      </c>
+      <c r="C23">
+        <v>5122</v>
+      </c>
+      <c r="D23">
+        <v>3.245509718570156</v>
+      </c>
+      <c r="E23">
+        <v>2.7997999999999999E-2</v>
+      </c>
+      <c r="F23">
+        <v>6.9694571763756011E-5</v>
+      </c>
+      <c r="G23">
+        <v>3.7094395741324111</v>
+      </c>
+      <c r="H23">
+        <v>-1.5528729908001491</v>
+      </c>
+      <c r="I23">
+        <v>-1.5488587139216301</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24">
+        <v>665</v>
+      </c>
+      <c r="C24">
+        <v>8165</v>
+      </c>
+      <c r="D24">
         <v>0</v>
       </c>
-      <c r="F13">
-        <v>2.3630000000000009E-2</v>
-      </c>
-      <c r="G13">
+      <c r="E24">
+        <v>2.2120000000000001E-2</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>3.9119561890726868</v>
+      </c>
+      <c r="H24">
+        <v>-1.655214877367339</v>
+      </c>
+      <c r="I24">
+        <v>-1.637786363408368</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25">
+        <v>65</v>
+      </c>
+      <c r="C25">
+        <v>50.3</v>
+      </c>
+      <c r="D25">
+        <v>1.932471072084766</v>
+      </c>
+      <c r="E25">
+        <v>0.22636899999999999</v>
+      </c>
+      <c r="F25">
+        <v>9.6514480721231095E-3</v>
+      </c>
+      <c r="G25">
+        <v>1.7015679850559271</v>
+      </c>
+      <c r="H25">
+        <v>-0.64518304767258239</v>
+      </c>
+      <c r="I25">
+        <v>-0.63426802337529631</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26">
+        <v>130</v>
+      </c>
+      <c r="C26">
+        <v>206.7</v>
+      </c>
+      <c r="D26">
+        <v>2.6459612829954851</v>
+      </c>
+      <c r="E26">
+        <v>0.125886</v>
+      </c>
+      <c r="F26">
+        <v>3.0218460877049621E-3</v>
+      </c>
+      <c r="G26">
+        <v>2.3153404766272878</v>
+      </c>
+      <c r="H26">
+        <v>-0.90002256584785312</v>
+      </c>
+      <c r="I26">
+        <v>-0.90375366549658631</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A27" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27">
+        <v>196</v>
+      </c>
+      <c r="C27">
+        <v>482.2</v>
+      </c>
+      <c r="D27">
+        <v>4.5504578524217392</v>
+      </c>
+      <c r="E27">
+        <v>8.7340000000000001E-2</v>
+      </c>
+      <c r="F27">
+        <v>1.83016331997387E-3</v>
+      </c>
+      <c r="G27">
+        <v>2.6832272060414351</v>
+      </c>
+      <c r="H27">
+        <v>-1.0587868124146791</v>
+      </c>
+      <c r="I27">
+        <v>-1.06527962644387</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A28" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28">
+        <v>262</v>
+      </c>
+      <c r="C28">
+        <v>861.6</v>
+      </c>
+      <c r="D28">
+        <v>7.7189521453512224</v>
+      </c>
+      <c r="E28">
+        <v>6.6927E-2</v>
+      </c>
+      <c r="F28">
+        <v>7.3840977783341984E-4</v>
+      </c>
+      <c r="G28">
+        <v>2.9353056902899248</v>
+      </c>
+      <c r="H28">
+        <v>-1.174398641792348</v>
+      </c>
+      <c r="I28">
+        <v>-1.1759583113402059</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29">
+        <v>327</v>
+      </c>
+      <c r="C29">
+        <v>1352.6</v>
+      </c>
+      <c r="D29">
+        <v>6.8737827205177844</v>
+      </c>
+      <c r="E29">
+        <v>5.5237000000000001E-2</v>
+      </c>
+      <c r="F29">
+        <v>4.2723672855013559E-4</v>
+      </c>
+      <c r="G29">
+        <v>3.1311693830893241</v>
+      </c>
+      <c r="H29">
+        <v>-1.2577699166036489</v>
+      </c>
+      <c r="I29">
+        <v>-1.26195508334796</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30">
+        <v>393</v>
+      </c>
+      <c r="C30">
+        <v>1946</v>
+      </c>
+      <c r="D30">
+        <v>11.99536947696439</v>
+      </c>
+      <c r="E30">
+        <v>4.6784000000000013E-2</v>
+      </c>
+      <c r="F30">
+        <v>2.1572204337990121E-4</v>
+      </c>
+      <c r="G30">
+        <v>3.2891428359323331</v>
+      </c>
+      <c r="H30">
+        <v>-1.329902649058252</v>
+      </c>
+      <c r="I30">
+        <v>-1.3313156004159781</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31">
+        <v>458</v>
+      </c>
+      <c r="C31">
+        <v>2656.6</v>
+      </c>
+      <c r="D31">
+        <v>6.4069406809247793</v>
+      </c>
+      <c r="E31">
+        <v>4.0791000000000001E-2</v>
+      </c>
+      <c r="F31">
+        <v>1.67573864310638E-4</v>
+      </c>
+      <c r="G31">
+        <v>3.4243261683092951</v>
+      </c>
+      <c r="H31">
+        <v>-1.38943564773124</v>
+      </c>
+      <c r="I31">
+        <v>-1.390669787235975</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A32" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32">
+        <v>524</v>
+      </c>
+      <c r="C32">
+        <v>3494.5</v>
+      </c>
+      <c r="D32">
+        <v>5.2667721508423817</v>
+      </c>
+      <c r="E32">
+        <v>3.6569999999999998E-2</v>
+      </c>
+      <c r="F32">
+        <v>8.2273257434532421E-5</v>
+      </c>
+      <c r="G32">
+        <v>3.5433850448098432</v>
+      </c>
+      <c r="H32">
+        <v>-1.4368750396619561</v>
+      </c>
+      <c r="I32">
+        <v>-1.4429442997379081</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A33" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B33">
+        <v>589</v>
+      </c>
+      <c r="C33">
+        <v>4403.3</v>
+      </c>
+      <c r="D33">
+        <v>3.2285187522040708</v>
+      </c>
+      <c r="E33">
+        <v>3.2891999999999998E-2</v>
+      </c>
+      <c r="F33">
+        <v>5.9363288318623168E-5</v>
+      </c>
+      <c r="G33">
+        <v>3.6437782752633301</v>
+      </c>
+      <c r="H33">
+        <v>-1.482909718412877</v>
+      </c>
+      <c r="I33">
+        <v>-1.487023391819934</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34">
+        <v>655</v>
+      </c>
+      <c r="C34">
+        <v>5438.6</v>
+      </c>
+      <c r="D34">
+        <v>5.8938762947467591</v>
+      </c>
+      <c r="E34">
+        <v>2.9750999999999989E-2</v>
+      </c>
+      <c r="F34">
+        <v>5.8849148016111702E-5</v>
+      </c>
+      <c r="G34">
+        <v>3.7354871183516791</v>
+      </c>
+      <c r="H34">
+        <v>-1.526498432046927</v>
+      </c>
+      <c r="I34">
+        <v>-1.527289478696183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A35" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35">
+        <v>665</v>
+      </c>
+      <c r="C35">
+        <v>8619</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>2.324E-2</v>
+      </c>
+      <c r="F35">
         <v>1.1564823173178709E-18</v>
       </c>
-      <c r="H13">
-        <v>3.9352552817840469</v>
-      </c>
-      <c r="I13">
-        <v>-1.6265362783676309</v>
-      </c>
-      <c r="J13">
-        <v>-1.6052597304157381</v>
-      </c>
-    </row>
-    <row r="14" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B14" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C14">
+      <c r="G35">
+        <v>3.9354568807116102</v>
+      </c>
+      <c r="H35">
+        <v>-1.6337638762817071</v>
+      </c>
+      <c r="I35">
+        <v>-1.6150890796141759</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A36" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36">
         <v>65</v>
       </c>
-      <c r="D14">
-        <v>47.8</v>
-      </c>
-      <c r="E14">
-        <v>1.481740718059525</v>
-      </c>
-      <c r="F14">
-        <v>0.20963699999999999</v>
-      </c>
-      <c r="G14">
-        <v>8.4001738143392648E-3</v>
-      </c>
-      <c r="H14">
-        <v>1.679427896612119</v>
-      </c>
-      <c r="I14">
-        <v>-0.67853206387484444</v>
-      </c>
-      <c r="J14">
-        <v>-0.65745448535624873</v>
-      </c>
-    </row>
-    <row r="15" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B15" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15">
+      <c r="C36">
+        <v>52.1</v>
+      </c>
+      <c r="D36">
+        <v>1.303414319734477</v>
+      </c>
+      <c r="E36">
+        <v>0.240152</v>
+      </c>
+      <c r="F36">
+        <v>8.7450770659205108E-3</v>
+      </c>
+      <c r="G36">
+        <v>1.716837723299524</v>
+      </c>
+      <c r="H36">
+        <v>-0.61951379217993485</v>
+      </c>
+      <c r="I36">
+        <v>-0.60123305459169774</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A37" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37">
         <v>130</v>
       </c>
-      <c r="D15">
-        <v>201.9</v>
-      </c>
-      <c r="E15">
-        <v>3.813572253587616</v>
-      </c>
-      <c r="F15">
-        <v>0.12109300000000001</v>
-      </c>
-      <c r="G15">
-        <v>3.5074850280824039E-3</v>
-      </c>
-      <c r="H15">
-        <v>2.3051363189436391</v>
-      </c>
-      <c r="I15">
-        <v>-0.91688096130979457</v>
-      </c>
-      <c r="J15">
-        <v>-0.93221109867613228</v>
-      </c>
-    </row>
-    <row r="16" spans="2:30" x14ac:dyDescent="0.2">
-      <c r="B16" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16">
+      <c r="C37">
+        <v>209.8</v>
+      </c>
+      <c r="D37">
+        <v>2.6364959911046908</v>
+      </c>
+      <c r="E37">
+        <v>0.13777800000000001</v>
+      </c>
+      <c r="F37">
+        <v>3.3789050823536831E-3</v>
+      </c>
+      <c r="G37">
+        <v>2.3218054838575388</v>
+      </c>
+      <c r="H37">
+        <v>-0.8608201238026838</v>
+      </c>
+      <c r="I37">
+        <v>-0.86610594476926028</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A38" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38">
         <v>196</v>
       </c>
-      <c r="D16">
-        <v>453</v>
-      </c>
-      <c r="E16">
-        <v>4.7539457296018854</v>
-      </c>
-      <c r="F16">
-        <v>8.2914000000000015E-2</v>
-      </c>
-      <c r="G16">
-        <v>1.122124176135005E-3</v>
-      </c>
-      <c r="H16">
-        <v>2.6560982020128319</v>
-      </c>
-      <c r="I16">
-        <v>-1.0813721327862229</v>
-      </c>
-      <c r="J16">
-        <v>-1.086322974039972</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B17" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17">
+      <c r="C38">
+        <v>468.5</v>
+      </c>
+      <c r="D38">
+        <v>5.497979426823802</v>
+      </c>
+      <c r="E38">
+        <v>9.8486999999999991E-2</v>
+      </c>
+      <c r="F38">
+        <v>1.65567646463781E-3</v>
+      </c>
+      <c r="G38">
+        <v>2.6707095952237969</v>
+      </c>
+      <c r="H38">
+        <v>-1.00662109133858</v>
+      </c>
+      <c r="I38">
+        <v>-1.018866548552795</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39">
         <v>262</v>
       </c>
-      <c r="D17">
-        <v>828.6</v>
-      </c>
-      <c r="E17">
-        <v>7.001904502823975</v>
-      </c>
-      <c r="F17">
-        <v>6.3450999999999994E-2</v>
-      </c>
-      <c r="G17">
-        <v>5.8089863334511436E-4</v>
-      </c>
-      <c r="H17">
-        <v>2.9183449289622749</v>
-      </c>
-      <c r="I17">
-        <v>-1.1975615289505279</v>
-      </c>
-      <c r="J17">
-        <v>-1.201478883692531</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B18" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18">
+      <c r="C39">
+        <v>827.9</v>
+      </c>
+      <c r="D39">
+        <v>7.2853734747551986</v>
+      </c>
+      <c r="E39">
+        <v>7.5895999999999991E-2</v>
+      </c>
+      <c r="F39">
+        <v>1.2227766217370469E-3</v>
+      </c>
+      <c r="G39">
+        <v>2.9179778825929081</v>
+      </c>
+      <c r="H39">
+        <v>-1.119781112427374</v>
+      </c>
+      <c r="I39">
+        <v>-1.1271279637797831</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A40" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B40">
         <v>327</v>
       </c>
-      <c r="D18">
-        <v>1287.8</v>
-      </c>
-      <c r="E18">
-        <v>4.2551929059287863</v>
-      </c>
-      <c r="F18">
-        <v>5.297799999999999E-2</v>
-      </c>
-      <c r="G18">
-        <v>4.0885694319651712E-4</v>
-      </c>
-      <c r="H18">
-        <v>3.109848420756105</v>
-      </c>
-      <c r="I18">
-        <v>-1.2759044410059239</v>
-      </c>
-      <c r="J18">
-        <v>-1.285570529203939</v>
-      </c>
-    </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B19" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19">
+      <c r="C40">
+        <v>1281.5999999999999</v>
+      </c>
+      <c r="D40">
+        <v>8.6976369715508852</v>
+      </c>
+      <c r="E40">
+        <v>6.2158999999999999E-2</v>
+      </c>
+      <c r="F40">
+        <v>9.4199368952828475E-4</v>
+      </c>
+      <c r="G40">
+        <v>3.107752498740163</v>
+      </c>
+      <c r="H40">
+        <v>-1.2064959809828071</v>
+      </c>
+      <c r="I40">
+        <v>-1.210216938661512</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A41" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41">
         <v>393</v>
       </c>
-      <c r="D19">
-        <v>1847</v>
-      </c>
-      <c r="E19">
-        <v>6.2307481270086829</v>
-      </c>
-      <c r="F19">
-        <v>4.4794E-2</v>
-      </c>
-      <c r="G19">
-        <v>2.9242358925975057E-4</v>
-      </c>
-      <c r="H19">
-        <v>3.2664668954402409</v>
-      </c>
-      <c r="I19">
-        <v>-1.3487801543366851</v>
-      </c>
-      <c r="J19">
-        <v>-1.3543437151668081</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B20" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C20">
+      <c r="C41">
+        <v>1852.8</v>
+      </c>
+      <c r="D41">
+        <v>6.5959583584697272</v>
+      </c>
+      <c r="E41">
+        <v>5.2861000000000012E-2</v>
+      </c>
+      <c r="F41">
+        <v>4.718484926329638E-4</v>
+      </c>
+      <c r="G41">
+        <v>3.2678285420473419</v>
+      </c>
+      <c r="H41">
+        <v>-1.2768646253440361</v>
+      </c>
+      <c r="I41">
+        <v>-1.280302994486789</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A42" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42">
         <v>458</v>
       </c>
-      <c r="D20">
-        <v>2522.6999999999998</v>
-      </c>
-      <c r="E20">
-        <v>6.4412731660751668</v>
-      </c>
-      <c r="F20">
-        <v>3.8827E-2</v>
-      </c>
-      <c r="G20">
-        <v>1.6180269191552729E-4</v>
-      </c>
-      <c r="H20">
-        <v>3.401865607199611</v>
-      </c>
-      <c r="I20">
-        <v>-1.4108661642769911</v>
-      </c>
-      <c r="J20">
-        <v>-1.413799030395358</v>
-      </c>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B21" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C21">
+      <c r="C42">
+        <v>2520.5</v>
+      </c>
+      <c r="D42">
+        <v>6.5357988545140113</v>
+      </c>
+      <c r="E42">
+        <v>4.6466E-2</v>
+      </c>
+      <c r="F42">
+        <v>3.3239267273646157E-4</v>
+      </c>
+      <c r="G42">
+        <v>3.4014867017741688</v>
+      </c>
+      <c r="H42">
+        <v>-1.332864711913158</v>
+      </c>
+      <c r="I42">
+        <v>-1.3388225146509769</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43">
         <v>524</v>
       </c>
-      <c r="D21">
-        <v>3294.9</v>
-      </c>
-      <c r="E21">
-        <v>4.3879886559156516</v>
-      </c>
-      <c r="F21">
-        <v>3.4486999999999997E-2</v>
-      </c>
-      <c r="G21">
-        <v>1.064273356698253E-4</v>
-      </c>
-      <c r="H21">
-        <v>3.5178422383208559</v>
-      </c>
-      <c r="I21">
-        <v>-1.4623445829626329</v>
-      </c>
-      <c r="J21">
-        <v>-1.4647258602954349</v>
-      </c>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B22" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C22">
+      <c r="C43">
+        <v>3331.1</v>
+      </c>
+      <c r="D43">
+        <v>13.673534859558281</v>
+      </c>
+      <c r="E43">
+        <v>4.0835000000000003E-2</v>
+      </c>
+      <c r="F43">
+        <v>1.570650962004112E-4</v>
+      </c>
+      <c r="G43">
+        <v>3.5225876704565038</v>
+      </c>
+      <c r="H43">
+        <v>-1.388967440075479</v>
+      </c>
+      <c r="I43">
+        <v>-1.391844122858009</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44">
         <v>589</v>
       </c>
-      <c r="D22">
-        <v>4152.6000000000004</v>
-      </c>
-      <c r="E22">
-        <v>5.2877216265609137</v>
-      </c>
-      <c r="F22">
-        <v>3.0827E-2</v>
-      </c>
-      <c r="G22">
-        <v>7.7374270773803059E-5</v>
-      </c>
-      <c r="H22">
-        <v>3.6183200996244</v>
-      </c>
-      <c r="I22">
-        <v>-1.511068737577747</v>
-      </c>
-      <c r="J22">
-        <v>-1.508846981092431</v>
-      </c>
-    </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B23" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C23">
+      <c r="C44">
+        <v>4192.1000000000004</v>
+      </c>
+      <c r="D44">
+        <v>11.21749625461146</v>
+      </c>
+      <c r="E44">
+        <v>3.6700999999999998E-2</v>
+      </c>
+      <c r="F44">
+        <v>4.61266372789805E-5</v>
+      </c>
+      <c r="G44">
+        <v>3.6224316339303919</v>
+      </c>
+      <c r="H44">
+        <v>-1.43532210227202</v>
+      </c>
+      <c r="I44">
+        <v>-1.4355587815494379</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45">
         <v>655</v>
       </c>
-      <c r="D23">
-        <v>5122</v>
-      </c>
-      <c r="E23">
-        <v>3.245509718570156</v>
-      </c>
-      <c r="F23">
-        <v>2.7997999999999999E-2</v>
-      </c>
-      <c r="G23">
-        <v>6.9694571763756011E-5</v>
-      </c>
-      <c r="H23">
-        <v>3.7094395741324111</v>
-      </c>
-      <c r="I23">
-        <v>-1.5528729908001491</v>
-      </c>
-      <c r="J23">
-        <v>-1.5488587139216301</v>
-      </c>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B24" s="27" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24">
+      <c r="C45">
+        <v>5196.1000000000004</v>
+      </c>
+      <c r="D45">
+        <v>11.75438452474461</v>
+      </c>
+      <c r="E45">
+        <v>3.3259999999999998E-2</v>
+      </c>
+      <c r="F45">
+        <v>2.0275875100993919E-5</v>
+      </c>
+      <c r="G45">
+        <v>3.715677500566942</v>
+      </c>
+      <c r="H45">
+        <v>-1.4780777551165001</v>
+      </c>
+      <c r="I45">
+        <v>-1.476384597077778</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46">
         <v>665</v>
       </c>
-      <c r="D24">
-        <v>8165</v>
-      </c>
-      <c r="E24">
+      <c r="C46">
+        <v>8269</v>
+      </c>
+      <c r="D46">
         <v>0</v>
       </c>
-      <c r="F24">
-        <v>2.2120000000000001E-2</v>
-      </c>
-      <c r="G24">
+      <c r="E46">
+        <v>2.5950000000000001E-2</v>
+      </c>
+      <c r="F46">
         <v>0</v>
       </c>
-      <c r="H24">
-        <v>3.9119561890726868</v>
-      </c>
-      <c r="I24">
-        <v>-1.655214877367339</v>
-      </c>
-      <c r="J24">
-        <v>-1.637786363408368</v>
-      </c>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B25" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25">
-        <v>65</v>
-      </c>
-      <c r="D25">
-        <v>50.3</v>
-      </c>
-      <c r="E25">
-        <v>1.932471072084766</v>
-      </c>
-      <c r="F25">
-        <v>0.22636899999999999</v>
-      </c>
-      <c r="G25">
-        <v>9.6514480721231095E-3</v>
-      </c>
-      <c r="H25">
-        <v>1.7015679850559271</v>
-      </c>
-      <c r="I25">
-        <v>-0.64518304767258239</v>
-      </c>
-      <c r="J25">
-        <v>-0.63426802337529631</v>
-      </c>
-    </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B26" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C26">
-        <v>130</v>
-      </c>
-      <c r="D26">
-        <v>206.7</v>
-      </c>
-      <c r="E26">
-        <v>2.6459612829954851</v>
-      </c>
-      <c r="F26">
-        <v>0.125886</v>
-      </c>
-      <c r="G26">
-        <v>3.0218460877049621E-3</v>
-      </c>
-      <c r="H26">
-        <v>2.3153404766272878</v>
-      </c>
-      <c r="I26">
-        <v>-0.90002256584785312</v>
-      </c>
-      <c r="J26">
-        <v>-0.90375366549658631</v>
-      </c>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B27" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C27">
-        <v>196</v>
-      </c>
-      <c r="D27">
-        <v>482.2</v>
-      </c>
-      <c r="E27">
-        <v>4.5504578524217392</v>
-      </c>
-      <c r="F27">
-        <v>8.7340000000000001E-2</v>
-      </c>
-      <c r="G27">
-        <v>1.83016331997387E-3</v>
-      </c>
-      <c r="H27">
-        <v>2.6832272060414351</v>
-      </c>
-      <c r="I27">
-        <v>-1.0587868124146791</v>
-      </c>
-      <c r="J27">
-        <v>-1.06527962644387</v>
-      </c>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B28" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28">
-        <v>262</v>
-      </c>
-      <c r="D28">
-        <v>861.6</v>
-      </c>
-      <c r="E28">
-        <v>7.7189521453512224</v>
-      </c>
-      <c r="F28">
-        <v>6.6927E-2</v>
-      </c>
-      <c r="G28">
-        <v>7.3840977783341984E-4</v>
-      </c>
-      <c r="H28">
-        <v>2.9353056902899248</v>
-      </c>
-      <c r="I28">
-        <v>-1.174398641792348</v>
-      </c>
-      <c r="J28">
-        <v>-1.1759583113402059</v>
-      </c>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B29" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29">
-        <v>327</v>
-      </c>
-      <c r="D29">
-        <v>1352.6</v>
-      </c>
-      <c r="E29">
-        <v>6.8737827205177844</v>
-      </c>
-      <c r="F29">
-        <v>5.5237000000000001E-2</v>
-      </c>
-      <c r="G29">
-        <v>4.2723672855013559E-4</v>
-      </c>
-      <c r="H29">
-        <v>3.1311693830893241</v>
-      </c>
-      <c r="I29">
-        <v>-1.2577699166036489</v>
-      </c>
-      <c r="J29">
-        <v>-1.26195508334796</v>
-      </c>
-    </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B30" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30">
-        <v>393</v>
-      </c>
-      <c r="D30">
-        <v>1946</v>
-      </c>
-      <c r="E30">
-        <v>11.99536947696439</v>
-      </c>
-      <c r="F30">
-        <v>4.6784000000000013E-2</v>
-      </c>
-      <c r="G30">
-        <v>2.1572204337990121E-4</v>
-      </c>
-      <c r="H30">
-        <v>3.2891428359323331</v>
-      </c>
-      <c r="I30">
-        <v>-1.329902649058252</v>
-      </c>
-      <c r="J30">
-        <v>-1.3313156004159781</v>
-      </c>
-    </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B31" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31">
-        <v>458</v>
-      </c>
-      <c r="D31">
-        <v>2656.6</v>
-      </c>
-      <c r="E31">
-        <v>6.4069406809247793</v>
-      </c>
-      <c r="F31">
-        <v>4.0791000000000001E-2</v>
-      </c>
-      <c r="G31">
-        <v>1.67573864310638E-4</v>
-      </c>
-      <c r="H31">
-        <v>3.4243261683092951</v>
-      </c>
-      <c r="I31">
-        <v>-1.38943564773124</v>
-      </c>
-      <c r="J31">
-        <v>-1.390669787235975</v>
-      </c>
-    </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B32" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32">
-        <v>524</v>
-      </c>
-      <c r="D32">
-        <v>3494.5</v>
-      </c>
-      <c r="E32">
-        <v>5.2667721508423817</v>
-      </c>
-      <c r="F32">
-        <v>3.6569999999999998E-2</v>
-      </c>
-      <c r="G32">
-        <v>8.2273257434532421E-5</v>
-      </c>
-      <c r="H32">
-        <v>3.5433850448098432</v>
-      </c>
-      <c r="I32">
-        <v>-1.4368750396619561</v>
-      </c>
-      <c r="J32">
-        <v>-1.4429442997379081</v>
-      </c>
-    </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B33" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C33">
-        <v>589</v>
-      </c>
-      <c r="D33">
-        <v>4403.3</v>
-      </c>
-      <c r="E33">
-        <v>3.2285187522040708</v>
-      </c>
-      <c r="F33">
-        <v>3.2891999999999998E-2</v>
-      </c>
-      <c r="G33">
-        <v>5.9363288318623168E-5</v>
-      </c>
-      <c r="H33">
-        <v>3.6437782752633301</v>
-      </c>
-      <c r="I33">
-        <v>-1.482909718412877</v>
-      </c>
-      <c r="J33">
-        <v>-1.487023391819934</v>
-      </c>
-    </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B34" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34">
-        <v>655</v>
-      </c>
-      <c r="D34">
-        <v>5438.6</v>
-      </c>
-      <c r="E34">
-        <v>5.8938762947467591</v>
-      </c>
-      <c r="F34">
-        <v>2.9750999999999989E-2</v>
-      </c>
-      <c r="G34">
-        <v>5.8849148016111702E-5</v>
-      </c>
-      <c r="H34">
-        <v>3.7354871183516791</v>
-      </c>
-      <c r="I34">
-        <v>-1.526498432046927</v>
-      </c>
-      <c r="J34">
-        <v>-1.527289478696183</v>
-      </c>
-    </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B35" s="27" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35">
-        <v>665</v>
-      </c>
-      <c r="D35">
-        <v>8619</v>
-      </c>
-      <c r="E35">
-        <v>0</v>
-      </c>
-      <c r="F35">
-        <v>2.324E-2</v>
-      </c>
-      <c r="G35">
-        <v>1.1564823173178709E-18</v>
-      </c>
-      <c r="H35">
-        <v>3.9354568807116102</v>
-      </c>
-      <c r="I35">
-        <v>-1.6337638762817071</v>
-      </c>
-      <c r="J35">
-        <v>-1.6150890796141759</v>
-      </c>
-    </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B36" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C36">
-        <v>65</v>
-      </c>
-      <c r="D36">
-        <v>52.1</v>
-      </c>
-      <c r="E36">
-        <v>1.303414319734477</v>
-      </c>
-      <c r="F36">
-        <v>0.240152</v>
-      </c>
-      <c r="G36">
-        <v>8.7450770659205108E-3</v>
-      </c>
-      <c r="H36">
-        <v>1.716837723299524</v>
-      </c>
-      <c r="I36">
-        <v>-0.61951379217993485</v>
-      </c>
-      <c r="J36">
-        <v>-0.60123305459169774</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B37" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C37">
-        <v>130</v>
-      </c>
-      <c r="D37">
-        <v>209.8</v>
-      </c>
-      <c r="E37">
-        <v>2.6364959911046908</v>
-      </c>
-      <c r="F37">
-        <v>0.13777800000000001</v>
-      </c>
-      <c r="G37">
-        <v>3.3789050823536831E-3</v>
-      </c>
-      <c r="H37">
-        <v>2.3218054838575388</v>
-      </c>
-      <c r="I37">
-        <v>-0.8608201238026838</v>
-      </c>
-      <c r="J37">
-        <v>-0.86610594476926028</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B38" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C38">
-        <v>196</v>
-      </c>
-      <c r="D38">
-        <v>468.5</v>
-      </c>
-      <c r="E38">
-        <v>5.497979426823802</v>
-      </c>
-      <c r="F38">
-        <v>9.8486999999999991E-2</v>
-      </c>
-      <c r="G38">
-        <v>1.65567646463781E-3</v>
-      </c>
-      <c r="H38">
-        <v>2.6707095952237969</v>
-      </c>
-      <c r="I38">
-        <v>-1.00662109133858</v>
-      </c>
-      <c r="J38">
-        <v>-1.018866548552795</v>
-      </c>
-    </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B39" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C39">
-        <v>262</v>
-      </c>
-      <c r="D39">
-        <v>827.9</v>
-      </c>
-      <c r="E39">
-        <v>7.2853734747551986</v>
-      </c>
-      <c r="F39">
-        <v>7.5895999999999991E-2</v>
-      </c>
-      <c r="G39">
-        <v>1.2227766217370469E-3</v>
-      </c>
-      <c r="H39">
-        <v>2.9179778825929081</v>
-      </c>
-      <c r="I39">
-        <v>-1.119781112427374</v>
-      </c>
-      <c r="J39">
-        <v>-1.1271279637797831</v>
-      </c>
-    </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B40" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C40">
-        <v>327</v>
-      </c>
-      <c r="D40">
-        <v>1281.5999999999999</v>
-      </c>
-      <c r="E40">
-        <v>8.6976369715508852</v>
-      </c>
-      <c r="F40">
-        <v>6.2158999999999999E-2</v>
-      </c>
-      <c r="G40">
-        <v>9.4199368952828475E-4</v>
-      </c>
-      <c r="H40">
-        <v>3.107752498740163</v>
-      </c>
-      <c r="I40">
-        <v>-1.2064959809828071</v>
-      </c>
-      <c r="J40">
-        <v>-1.210216938661512</v>
-      </c>
-    </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B41" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C41">
-        <v>393</v>
-      </c>
-      <c r="D41">
-        <v>1852.8</v>
-      </c>
-      <c r="E41">
-        <v>6.5959583584697272</v>
-      </c>
-      <c r="F41">
-        <v>5.2861000000000012E-2</v>
-      </c>
-      <c r="G41">
-        <v>4.718484926329638E-4</v>
-      </c>
-      <c r="H41">
-        <v>3.2678285420473419</v>
-      </c>
-      <c r="I41">
-        <v>-1.2768646253440361</v>
-      </c>
-      <c r="J41">
-        <v>-1.280302994486789</v>
-      </c>
-    </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B42" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42">
-        <v>458</v>
-      </c>
-      <c r="D42">
-        <v>2520.5</v>
-      </c>
-      <c r="E42">
-        <v>6.5357988545140113</v>
-      </c>
-      <c r="F42">
-        <v>4.6466E-2</v>
-      </c>
-      <c r="G42">
-        <v>3.3239267273646157E-4</v>
-      </c>
-      <c r="H42">
-        <v>3.4014867017741688</v>
-      </c>
-      <c r="I42">
-        <v>-1.332864711913158</v>
-      </c>
-      <c r="J42">
-        <v>-1.3388225146509769</v>
-      </c>
-    </row>
-    <row r="43" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B43" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C43">
-        <v>524</v>
-      </c>
-      <c r="D43">
-        <v>3331.1</v>
-      </c>
-      <c r="E43">
-        <v>13.673534859558281</v>
-      </c>
-      <c r="F43">
-        <v>4.0835000000000003E-2</v>
-      </c>
-      <c r="G43">
-        <v>1.570650962004112E-4</v>
-      </c>
-      <c r="H43">
-        <v>3.5225876704565038</v>
-      </c>
-      <c r="I43">
-        <v>-1.388967440075479</v>
-      </c>
-      <c r="J43">
-        <v>-1.391844122858009</v>
-      </c>
-    </row>
-    <row r="44" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B44" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C44">
-        <v>589</v>
-      </c>
-      <c r="D44">
-        <v>4192.1000000000004</v>
-      </c>
-      <c r="E44">
-        <v>11.21749625461146</v>
-      </c>
-      <c r="F44">
-        <v>3.6700999999999998E-2</v>
-      </c>
-      <c r="G44">
-        <v>4.61266372789805E-5</v>
-      </c>
-      <c r="H44">
-        <v>3.6224316339303919</v>
-      </c>
-      <c r="I44">
-        <v>-1.43532210227202</v>
-      </c>
-      <c r="J44">
-        <v>-1.4355587815494379</v>
-      </c>
-    </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B45" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C45">
-        <v>655</v>
-      </c>
-      <c r="D45">
-        <v>5196.1000000000004</v>
-      </c>
-      <c r="E45">
-        <v>11.75438452474461</v>
-      </c>
-      <c r="F45">
-        <v>3.3259999999999998E-2</v>
-      </c>
-      <c r="G45">
-        <v>2.0275875100993919E-5</v>
-      </c>
-      <c r="H45">
-        <v>3.715677500566942</v>
-      </c>
-      <c r="I45">
-        <v>-1.4780777551165001</v>
-      </c>
-      <c r="J45">
-        <v>-1.476384597077778</v>
-      </c>
-    </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B46" s="27" t="s">
-        <v>7</v>
-      </c>
-      <c r="C46">
-        <v>665</v>
-      </c>
-      <c r="D46">
-        <v>8269</v>
-      </c>
-      <c r="E46">
-        <v>0</v>
-      </c>
-      <c r="F46">
-        <v>2.5950000000000001E-2</v>
-      </c>
       <c r="G46">
-        <v>0</v>
+        <v>3.9174529919296641</v>
       </c>
       <c r="H46">
-        <v>3.9174529919296641</v>
+        <v>-1.5858626378155229</v>
       </c>
       <c r="I46">
-        <v>-1.5858626378155229</v>
-      </c>
-      <c r="J46">
         <v>-1.564727912290055</v>
       </c>
     </row>
@@ -13133,7 +12897,9 @@
       <c r="I1" s="27"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="27"/>
+      <c r="A2" s="31" t="s">
+        <v>25</v>
+      </c>
       <c r="B2" s="28" t="s">
         <v>26</v>
       </c>
@@ -14457,7 +14223,9 @@
       <c r="I1" s="27"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="27"/>
+      <c r="A2" s="31" t="s">
+        <v>25</v>
+      </c>
       <c r="B2" s="28" t="s">
         <v>26</v>
       </c>
@@ -15050,7 +14818,7 @@
       <c r="E22" s="22">
         <v>3.0827E-2</v>
       </c>
-      <c r="F22" s="31">
+      <c r="F22" s="22">
         <v>7.7399999999999998E-5</v>
       </c>
       <c r="G22" s="22">
@@ -15079,7 +14847,7 @@
       <c r="E23" s="22">
         <v>2.7997999999999999E-2</v>
       </c>
-      <c r="F23" s="31">
+      <c r="F23" s="22">
         <v>6.97E-5</v>
       </c>
       <c r="G23" s="22">

</xml_diff>

<commit_message>
version 3.5.0: - average of 90% image (what about length < num_patches) - Histogram 3D RunTime warning
</commit_message>
<xml_diff>
--- a/results/SamChigome/Analysis_v2.xlsx
+++ b/results/SamChigome/Analysis_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owuor\owProjects\StructuralGT\results\SamChigome\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E64A81BF-246E-4A4A-AF6E-3BC8D5A88E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A78CFBDA-658D-470D-8EF2-509AD72E95B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="105" windowWidth="14610" windowHeight="15480" firstSheet="6" activeTab="7" xr2:uid="{E8351862-8131-4AC1-82A9-213539580791}"/>
+    <workbookView xWindow="12825" yWindow="0" windowWidth="17445" windowHeight="14775" firstSheet="5" activeTab="7" xr2:uid="{E8351862-8131-4AC1-82A9-213539580791}"/>
   </bookViews>
   <sheets>
     <sheet name="SGT Descriptors" sheetId="2" r:id="rId1"/>
@@ -6103,7 +6103,7 @@
   <dimension ref="A2:K46"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.85546875" style="21" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" style="21" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" customWidth="1"/>
     <col min="4" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="14.140625" customWidth="1"/>
@@ -6147,55 +6147,319 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
+      <c r="C3">
+        <v>53.9</v>
+      </c>
+      <c r="D3">
+        <v>1.9174636024359539</v>
+      </c>
+      <c r="E3">
+        <v>84.8</v>
+      </c>
+      <c r="F3">
+        <v>3.5017455964450388</v>
+      </c>
+      <c r="G3">
+        <v>1.731588765186739</v>
+      </c>
+      <c r="H3">
+        <v>1.9283958522567139</v>
+      </c>
+      <c r="I3">
+        <v>1.9407258214499949</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
+      <c r="B4">
+        <v>131</v>
+      </c>
+      <c r="C4">
+        <v>218.7</v>
+      </c>
+      <c r="D4">
+        <v>4.1794470660337089</v>
+      </c>
+      <c r="E4">
+        <v>372.1</v>
+      </c>
+      <c r="F4">
+        <v>7.5357665686894642</v>
+      </c>
+      <c r="G4">
+        <v>2.3398487830376369</v>
+      </c>
+      <c r="H4">
+        <v>2.5706596700215338</v>
+      </c>
+      <c r="I4">
+        <v>2.562815299227351</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>196</v>
+      </c>
+      <c r="C5">
+        <v>480.2</v>
+      </c>
+      <c r="D5">
+        <v>2.48461935381123</v>
+      </c>
+      <c r="E5">
+        <v>822.9</v>
+      </c>
+      <c r="F5">
+        <v>6.4557467938780464</v>
+      </c>
+      <c r="G5">
+        <v>2.6814221557210089</v>
+      </c>
+      <c r="H5">
+        <v>2.9153470623241922</v>
+      </c>
+      <c r="I5">
+        <v>2.9121547178957279</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>262</v>
+      </c>
+      <c r="C6">
+        <v>862.5</v>
+      </c>
+      <c r="D6">
+        <v>4.7755162606314672</v>
+      </c>
+      <c r="E6">
+        <v>1504.5</v>
+      </c>
+      <c r="F6">
+        <v>11.744738774825469</v>
+      </c>
+      <c r="G6">
+        <v>2.9357591037453119</v>
+      </c>
+      <c r="H6">
+        <v>3.1773921920760988</v>
+      </c>
+      <c r="I6">
+        <v>3.172274295925777</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
+      <c r="B7">
+        <v>328</v>
+      </c>
+      <c r="C7">
+        <v>1345.8</v>
+      </c>
+      <c r="D7">
+        <v>5.6819402007100033</v>
+      </c>
+      <c r="E7">
+        <v>2365.4</v>
+      </c>
+      <c r="F7">
+        <v>11.50091783776891</v>
+      </c>
+      <c r="G7">
+        <v>3.1289805239666109</v>
+      </c>
+      <c r="H7">
+        <v>3.37390459247497</v>
+      </c>
+      <c r="I7">
+        <v>3.3698888174679968</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
+      <c r="B8">
+        <v>393</v>
+      </c>
+      <c r="C8">
+        <v>1950.4</v>
+      </c>
+      <c r="D8">
+        <v>5.619806244188692</v>
+      </c>
+      <c r="E8">
+        <v>3444.2</v>
+      </c>
+      <c r="F8">
+        <v>12.579348154813109</v>
+      </c>
+      <c r="G8">
+        <v>3.2901236882743068</v>
+      </c>
+      <c r="H8">
+        <v>3.5370883624025349</v>
+      </c>
+      <c r="I8">
+        <v>3.5346957486974269</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
+      <c r="B9">
+        <v>459</v>
+      </c>
+      <c r="C9">
+        <v>2662.6</v>
+      </c>
+      <c r="D9">
+        <v>4.9959983987187186</v>
+      </c>
+      <c r="E9">
+        <v>4736.3999999999996</v>
+      </c>
+      <c r="F9">
+        <v>12.070349345952391</v>
+      </c>
+      <c r="G9">
+        <v>3.4253059276703191</v>
+      </c>
+      <c r="H9">
+        <v>3.6754483724431402</v>
+      </c>
+      <c r="I9">
+        <v>3.6729515048586889</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
+      <c r="B10">
+        <v>524</v>
+      </c>
+      <c r="C10">
+        <v>3464.1</v>
+      </c>
+      <c r="D10">
+        <v>4.1000000000000014</v>
+      </c>
+      <c r="E10">
+        <v>6184.1</v>
+      </c>
+      <c r="F10">
+        <v>11.518535786577511</v>
+      </c>
+      <c r="G10">
+        <v>3.5395904205339161</v>
+      </c>
+      <c r="H10">
+        <v>3.791276503726738</v>
+      </c>
+      <c r="I10">
+        <v>3.7898343812554618</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
+      <c r="B11">
+        <v>590</v>
+      </c>
+      <c r="C11">
+        <v>4413.3</v>
+      </c>
+      <c r="D11">
+        <v>7.7172965905598483</v>
+      </c>
+      <c r="E11">
+        <v>7860.5</v>
+      </c>
+      <c r="F11">
+        <v>26.073081052218502</v>
+      </c>
+      <c r="G11">
+        <v>3.644763450201828</v>
+      </c>
+      <c r="H11">
+        <v>3.8954501720361669</v>
+      </c>
+      <c r="I11">
+        <v>3.897398635328154</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
+      <c r="B12">
+        <v>656</v>
+      </c>
+      <c r="C12">
+        <v>5475.3</v>
+      </c>
+      <c r="D12">
+        <v>2.4857370916669539</v>
+      </c>
+      <c r="E12">
+        <v>9784.2000000000007</v>
+      </c>
+      <c r="F12">
+        <v>5.6111001100002156</v>
+      </c>
+      <c r="G12">
+        <v>3.7384079198181208</v>
+      </c>
+      <c r="H12">
+        <v>3.9905253215843031</v>
+      </c>
+      <c r="I12">
+        <v>3.9931722148676481</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>4</v>
+      </c>
+      <c r="B13">
+        <v>666</v>
+      </c>
+      <c r="C13">
+        <v>8615</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>15308</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>3.9352552817840469</v>
+      </c>
+      <c r="H13">
+        <v>4.1849184535524619</v>
+      </c>
+      <c r="I13">
+        <v>4.1944951179246281</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -7205,55 +7469,319 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
+      <c r="C3">
+        <v>53.9</v>
+      </c>
+      <c r="D3">
+        <v>1.9174636024359539</v>
+      </c>
+      <c r="E3">
+        <v>3.1450900000000002</v>
+      </c>
+      <c r="F3">
+        <v>6.3120149714651325E-2</v>
+      </c>
+      <c r="G3">
+        <v>1.731588765186739</v>
+      </c>
+      <c r="H3">
+        <v>0.49763307774444049</v>
+      </c>
+      <c r="I3">
+        <v>0.51006056698685842</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
+      <c r="B4">
+        <v>131</v>
+      </c>
+      <c r="C4">
+        <v>218.7</v>
+      </c>
+      <c r="D4">
+        <v>4.1794470660337089</v>
+      </c>
+      <c r="E4">
+        <v>3.402806</v>
+      </c>
+      <c r="F4">
+        <v>2.2077212092512441E-2</v>
+      </c>
+      <c r="G4">
+        <v>2.3398487830376369</v>
+      </c>
+      <c r="H4">
+        <v>0.53183718990358098</v>
+      </c>
+      <c r="I4">
+        <v>0.52392876133226562</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>196</v>
+      </c>
+      <c r="C5">
+        <v>480.2</v>
+      </c>
+      <c r="D5">
+        <v>2.48461935381123</v>
+      </c>
+      <c r="E5">
+        <v>3.427442000000001</v>
+      </c>
+      <c r="F5">
+        <v>2.2532037625469119E-2</v>
+      </c>
+      <c r="G5">
+        <v>2.6814221557210089</v>
+      </c>
+      <c r="H5">
+        <v>0.53497011428778607</v>
+      </c>
+      <c r="I5">
+        <v>0.53171655894606573</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>262</v>
+      </c>
+      <c r="C6">
+        <v>862.5</v>
+      </c>
+      <c r="D6">
+        <v>4.7755162606314672</v>
+      </c>
+      <c r="E6">
+        <v>3.4885860000000002</v>
+      </c>
+      <c r="F6">
+        <v>1.6858418681609609E-2</v>
+      </c>
+      <c r="G6">
+        <v>2.9357591037453119</v>
+      </c>
+      <c r="H6">
+        <v>0.54264943359725393</v>
+      </c>
+      <c r="I6">
+        <v>0.53751538530470266</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
+      <c r="B7">
+        <v>328</v>
+      </c>
+      <c r="C7">
+        <v>1345.8</v>
+      </c>
+      <c r="D7">
+        <v>5.6819402007100033</v>
+      </c>
+      <c r="E7">
+        <v>3.515368</v>
+      </c>
+      <c r="F7">
+        <v>1.319026701776729E-2</v>
+      </c>
+      <c r="G7">
+        <v>3.1289805239666109</v>
+      </c>
+      <c r="H7">
+        <v>0.54597079507527202</v>
+      </c>
+      <c r="I7">
+        <v>0.5419207910994025</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
+      <c r="B8">
+        <v>393</v>
+      </c>
+      <c r="C8">
+        <v>1950.4</v>
+      </c>
+      <c r="D8">
+        <v>5.619806244188692</v>
+      </c>
+      <c r="E8">
+        <v>3.5318290000000001</v>
+      </c>
+      <c r="F8">
+        <v>9.6383914575456486E-3</v>
+      </c>
+      <c r="G8">
+        <v>3.2901236882743068</v>
+      </c>
+      <c r="H8">
+        <v>0.54799966824805668</v>
+      </c>
+      <c r="I8">
+        <v>0.54559481972937696</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
+      <c r="B9">
+        <v>459</v>
+      </c>
+      <c r="C9">
+        <v>2662.6</v>
+      </c>
+      <c r="D9">
+        <v>4.9959983987187186</v>
+      </c>
+      <c r="E9">
+        <v>3.5577209999999999</v>
+      </c>
+      <c r="F9">
+        <v>5.8242953698757049E-3</v>
+      </c>
+      <c r="G9">
+        <v>3.4253059276703191</v>
+      </c>
+      <c r="H9">
+        <v>0.55117188728039912</v>
+      </c>
+      <c r="I9">
+        <v>0.5486769449931993</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
+      <c r="B10">
+        <v>524</v>
+      </c>
+      <c r="C10">
+        <v>3464.1</v>
+      </c>
+      <c r="D10">
+        <v>4.1000000000000014</v>
+      </c>
+      <c r="E10">
+        <v>3.570395</v>
+      </c>
+      <c r="F10">
+        <v>5.2432837992998109E-3</v>
+      </c>
+      <c r="G10">
+        <v>3.5395904205339161</v>
+      </c>
+      <c r="H10">
+        <v>0.55271626564461451</v>
+      </c>
+      <c r="I10">
+        <v>0.55128260624198311</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
+      <c r="B11">
+        <v>590</v>
+      </c>
+      <c r="C11">
+        <v>4413.3</v>
+      </c>
+      <c r="D11">
+        <v>7.7172965905598483</v>
+      </c>
+      <c r="E11">
+        <v>3.5621109999999998</v>
+      </c>
+      <c r="F11">
+        <v>6.4844203801624738E-3</v>
+      </c>
+      <c r="G11">
+        <v>3.644763450201828</v>
+      </c>
+      <c r="H11">
+        <v>0.55170744851756504</v>
+      </c>
+      <c r="I11">
+        <v>0.5536805281380881</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
+      <c r="B12">
+        <v>656</v>
+      </c>
+      <c r="C12">
+        <v>5475.3</v>
+      </c>
+      <c r="D12">
+        <v>2.4857370916669539</v>
+      </c>
+      <c r="E12">
+        <v>3.573941</v>
+      </c>
+      <c r="F12">
+        <v>1.5668258429775029E-3</v>
+      </c>
+      <c r="G12">
+        <v>3.7384079198181208</v>
+      </c>
+      <c r="H12">
+        <v>0.55314737872756292</v>
+      </c>
+      <c r="I12">
+        <v>0.55581560140593145</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>4</v>
+      </c>
+      <c r="B13">
+        <v>666</v>
+      </c>
+      <c r="C13">
+        <v>8615</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>3.5537999999999998</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>3.9352552817840469</v>
+      </c>
+      <c r="H13">
+        <v>0.55069298302458713</v>
+      </c>
+      <c r="I13">
+        <v>0.56030367787324464</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -8273,55 +8801,319 @@
       <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
+      <c r="C3">
+        <v>53.9</v>
+      </c>
+      <c r="D3">
+        <v>1.9174636024359539</v>
+      </c>
+      <c r="E3">
+        <v>10.8</v>
+      </c>
+      <c r="F3">
+        <v>0.41633319989322648</v>
+      </c>
+      <c r="G3">
+        <v>1.731588765186739</v>
+      </c>
+      <c r="H3">
+        <v>1.0334237554869501</v>
+      </c>
+      <c r="I3">
+        <v>1.019491982774134</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B4">
+        <v>131</v>
+      </c>
+      <c r="C4">
+        <v>218.7</v>
+      </c>
+      <c r="D4">
+        <v>4.1794470660337089</v>
+      </c>
+      <c r="E4">
+        <v>19.7</v>
+      </c>
+      <c r="F4">
+        <v>0.39581140290126388</v>
+      </c>
+      <c r="G4">
+        <v>2.3398487830376369</v>
+      </c>
+      <c r="H4">
+        <v>1.2944662261615929</v>
+      </c>
+      <c r="I4">
+        <v>1.3033313549351371</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>196</v>
+      </c>
+      <c r="C5">
+        <v>480.2</v>
+      </c>
+      <c r="D5">
+        <v>2.48461935381123</v>
+      </c>
+      <c r="E5">
+        <v>28.9</v>
+      </c>
+      <c r="F5">
+        <v>0.67412494720522276</v>
+      </c>
+      <c r="G5">
+        <v>2.6814221557210089</v>
+      </c>
+      <c r="H5">
+        <v>1.460897842756548</v>
+      </c>
+      <c r="I5">
+        <v>1.462723668754998</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>262</v>
+      </c>
+      <c r="C6">
+        <v>862.5</v>
+      </c>
+      <c r="D6">
+        <v>4.7755162606314672</v>
+      </c>
+      <c r="E6">
+        <v>37.700000000000003</v>
+      </c>
+      <c r="F6">
+        <v>0.73105707331537684</v>
+      </c>
+      <c r="G6">
+        <v>2.9357591037453119</v>
+      </c>
+      <c r="H6">
+        <v>1.576341350205793</v>
+      </c>
+      <c r="I6">
+        <v>1.581407845794331</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B7">
+        <v>328</v>
+      </c>
+      <c r="C7">
+        <v>1345.8</v>
+      </c>
+      <c r="D7">
+        <v>5.6819402007100033</v>
+      </c>
+      <c r="E7">
+        <v>46.2</v>
+      </c>
+      <c r="F7">
+        <v>0.5925462944877059</v>
+      </c>
+      <c r="G7">
+        <v>3.1289805239666109</v>
+      </c>
+      <c r="H7">
+        <v>1.664641975556125</v>
+      </c>
+      <c r="I7">
+        <v>1.671572980759876</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B8">
+        <v>393</v>
+      </c>
+      <c r="C8">
+        <v>1950.4</v>
+      </c>
+      <c r="D8">
+        <v>5.619806244188692</v>
+      </c>
+      <c r="E8">
+        <v>57.4</v>
+      </c>
+      <c r="F8">
+        <v>0.68637534273246648</v>
+      </c>
+      <c r="G8">
+        <v>3.2901236882743068</v>
+      </c>
+      <c r="H8">
+        <v>1.758911892397973</v>
+      </c>
+      <c r="I8">
+        <v>1.746769070002661</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B9">
+        <v>459</v>
+      </c>
+      <c r="C9">
+        <v>2662.6</v>
+      </c>
+      <c r="D9">
+        <v>4.9959983987187186</v>
+      </c>
+      <c r="E9">
+        <v>63.1</v>
+      </c>
+      <c r="F9">
+        <v>0.73711147958319934</v>
+      </c>
+      <c r="G9">
+        <v>3.4253059276703191</v>
+      </c>
+      <c r="H9">
+        <v>1.8000293592441341</v>
+      </c>
+      <c r="I9">
+        <v>1.809850714088115</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B10">
+        <v>524</v>
+      </c>
+      <c r="C10">
+        <v>3464.1</v>
+      </c>
+      <c r="D10">
+        <v>4.1000000000000014</v>
+      </c>
+      <c r="E10">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="F10">
+        <v>0.74833147735478822</v>
+      </c>
+      <c r="G10">
+        <v>3.5395904205339161</v>
+      </c>
+      <c r="H10">
+        <v>1.854913022307856</v>
+      </c>
+      <c r="I10">
+        <v>1.8631806022118711</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B11">
+        <v>590</v>
+      </c>
+      <c r="C11">
+        <v>4413.3</v>
+      </c>
+      <c r="D11">
+        <v>7.7172965905598483</v>
+      </c>
+      <c r="E11">
+        <v>80.5</v>
+      </c>
+      <c r="F11">
+        <v>0.42817441928883759</v>
+      </c>
+      <c r="G11">
+        <v>3.644763450201828</v>
+      </c>
+      <c r="H11">
+        <v>1.905795880367869</v>
+      </c>
+      <c r="I11">
+        <v>1.9122587034072851</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B12">
+        <v>656</v>
+      </c>
+      <c r="C12">
+        <v>5475.3</v>
+      </c>
+      <c r="D12">
+        <v>2.4857370916669539</v>
+      </c>
+      <c r="E12">
+        <v>89</v>
+      </c>
+      <c r="F12">
+        <v>0.59628479399994383</v>
+      </c>
+      <c r="G12">
+        <v>3.7384079198181208</v>
+      </c>
+      <c r="H12">
+        <v>1.949390006644913</v>
+      </c>
+      <c r="I12">
+        <v>1.955957099951827</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>4</v>
+      </c>
+      <c r="B13">
+        <v>666</v>
+      </c>
+      <c r="C13">
+        <v>8615</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>119</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>3.9352552817840469</v>
+      </c>
+      <c r="H13">
+        <v>2.075546961392531</v>
+      </c>
+      <c r="I13">
+        <v>2.0478142498420469</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -9343,54 +10135,262 @@
       <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
+      <c r="C3">
+        <v>53.9</v>
+      </c>
+      <c r="D3">
+        <v>1.9174636024359539</v>
+      </c>
+      <c r="E3">
+        <v>6.0070999999999999E-2</v>
+      </c>
+      <c r="F3">
+        <v>2.236675832072627E-3</v>
+      </c>
+      <c r="G3">
+        <v>1.731588765186739</v>
+      </c>
+      <c r="H3">
+        <v>-1.2213351383062321</v>
+      </c>
+      <c r="I3">
+        <v>-1.21265489211005</v>
+      </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B4">
+        <v>131</v>
+      </c>
+      <c r="C4">
+        <v>218.7</v>
+      </c>
+      <c r="D4">
+        <v>4.1794470660337089</v>
+      </c>
+      <c r="E4">
+        <v>1.5685999999999999E-2</v>
+      </c>
+      <c r="F4">
+        <v>3.3205488167537082E-4</v>
+      </c>
+      <c r="G4">
+        <v>2.3398487830376369</v>
+      </c>
+      <c r="H4">
+        <v>-1.8044877893259279</v>
+      </c>
+      <c r="I4">
+        <v>-1.810313726683723</v>
+      </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>196</v>
+      </c>
+      <c r="C5">
+        <v>480.2</v>
+      </c>
+      <c r="D5">
+        <v>2.48461935381123</v>
+      </c>
+      <c r="E5">
+        <v>7.1540000000000006E-3</v>
+      </c>
+      <c r="F5">
+        <v>6.305553108173783E-5</v>
+      </c>
+      <c r="G5">
+        <v>2.6814221557210089</v>
+      </c>
+      <c r="H5">
+        <v>-2.145451064187049</v>
+      </c>
+      <c r="I5">
+        <v>-2.1459339184573412</v>
+      </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>262</v>
+      </c>
+      <c r="C6">
+        <v>862.5</v>
+      </c>
+      <c r="D6">
+        <v>4.7755162606314672</v>
+      </c>
+      <c r="E6">
+        <v>4.0489999999999996E-3</v>
+      </c>
+      <c r="F6">
+        <v>2.8301943396169769E-5</v>
+      </c>
+      <c r="G6">
+        <v>2.9357591037453119</v>
+      </c>
+      <c r="H6">
+        <v>-2.392652223231587</v>
+      </c>
+      <c r="I6">
+        <v>-2.3958381033194329</v>
+      </c>
     </row>
     <row r="7" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
-      <c r="I7"/>
+      <c r="B7">
+        <v>328</v>
+      </c>
+      <c r="C7">
+        <v>1345.8</v>
+      </c>
+      <c r="D7">
+        <v>5.6819402007100033</v>
+      </c>
+      <c r="E7">
+        <v>2.614E-3</v>
+      </c>
+      <c r="F7">
+        <v>1.6411378166788241E-5</v>
+      </c>
+      <c r="G7">
+        <v>3.1289805239666109</v>
+      </c>
+      <c r="H7">
+        <v>-2.5826944167554751</v>
+      </c>
+      <c r="I7">
+        <v>-2.5856919247692578</v>
+      </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B8">
+        <v>393</v>
+      </c>
+      <c r="C8">
+        <v>1950.4</v>
+      </c>
+      <c r="D8">
+        <v>5.619806244188692</v>
+      </c>
+      <c r="E8">
+        <v>1.8140000000000001E-3</v>
+      </c>
+      <c r="F8">
+        <v>7.7746025264604083E-6</v>
+      </c>
+      <c r="G8">
+        <v>3.2901236882743068</v>
+      </c>
+      <c r="H8">
+        <v>-2.7413627172759241</v>
+      </c>
+      <c r="I8">
+        <v>-2.744026572704739</v>
+      </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B9">
+        <v>459</v>
+      </c>
+      <c r="C9">
+        <v>2662.6</v>
+      </c>
+      <c r="D9">
+        <v>4.9959983987187186</v>
+      </c>
+      <c r="E9">
+        <v>1.3370000000000001E-3</v>
+      </c>
+      <c r="F9">
+        <v>3.349958540373639E-6</v>
+      </c>
+      <c r="G9">
+        <v>3.4253059276703191</v>
+      </c>
+      <c r="H9">
+        <v>-2.873868592738015</v>
+      </c>
+      <c r="I9">
+        <v>-2.8768527609818122</v>
+      </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B10">
+        <v>524</v>
+      </c>
+      <c r="C10">
+        <v>3464.1</v>
+      </c>
+      <c r="D10">
+        <v>4.1000000000000014</v>
+      </c>
+      <c r="E10">
+        <v>1.031E-3</v>
+      </c>
+      <c r="F10">
+        <v>1.7950549357114819E-6</v>
+      </c>
+      <c r="G10">
+        <v>3.5395904205339161</v>
+      </c>
+      <c r="H10">
+        <v>-2.9867413347164828</v>
+      </c>
+      <c r="I10">
+        <v>-2.989145423346879</v>
+      </c>
       <c r="K10" s="1"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>4</v>
+      </c>
+      <c r="B11">
+        <v>590</v>
+      </c>
+      <c r="C11">
+        <v>4413.3</v>
+      </c>
+      <c r="D11">
+        <v>7.7172965905598483</v>
+      </c>
+      <c r="E11">
+        <v>8.070000000000001E-4</v>
+      </c>
+      <c r="F11">
+        <v>1.5275252316519341E-6</v>
+      </c>
+      <c r="G11">
+        <v>3.644763450201828</v>
+      </c>
+      <c r="H11">
+        <v>-3.0931264652779289</v>
+      </c>
+      <c r="I11">
+        <v>-3.0924854235033838</v>
       </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
@@ -9407,10 +10407,58 @@
       <c r="A12" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B12">
+        <v>656</v>
+      </c>
+      <c r="C12">
+        <v>5475.3</v>
+      </c>
+      <c r="D12">
+        <v>2.4857370916669539</v>
+      </c>
+      <c r="E12">
+        <v>6.5099999999999989E-4</v>
+      </c>
+      <c r="F12">
+        <v>1.0000000000000021E-6</v>
+      </c>
+      <c r="G12">
+        <v>3.7384079198181208</v>
+      </c>
+      <c r="H12">
+        <v>-3.1864190114318078</v>
+      </c>
+      <c r="I12">
+        <v>-3.184497791458929</v>
+      </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>4</v>
+      </c>
+      <c r="B13">
+        <v>666</v>
+      </c>
+      <c r="C13">
+        <v>8615</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>4.0999999999999988E-4</v>
+      </c>
+      <c r="F13">
+        <v>1.807003620809174E-20</v>
+      </c>
+      <c r="G13">
+        <v>3.9352552817840469</v>
+      </c>
+      <c r="H13">
+        <v>-3.387216143280265</v>
+      </c>
+      <c r="I13">
+        <v>-3.3779143591911449</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
@@ -10483,14 +11531,30 @@
       <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
-      <c r="E3"/>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
-      <c r="I3"/>
+      <c r="B3">
+        <v>65</v>
+      </c>
+      <c r="C3">
+        <v>53.9</v>
+      </c>
+      <c r="D3">
+        <v>1.9174636024359539</v>
+      </c>
+      <c r="E3">
+        <v>7.0045999999999997E-2</v>
+      </c>
+      <c r="F3">
+        <v>2.3100174121517881E-3</v>
+      </c>
+      <c r="G3">
+        <v>1.731588765186739</v>
+      </c>
+      <c r="H3">
+        <v>-1.154616660200158</v>
+      </c>
+      <c r="I3">
+        <v>-1.157428682441286</v>
+      </c>
       <c r="J3" s="15"/>
       <c r="K3" s="15"/>
       <c r="L3" s="15"/>
@@ -10516,14 +11580,30 @@
       <c r="A4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
-      <c r="E4"/>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
+      <c r="B4">
+        <v>131</v>
+      </c>
+      <c r="C4">
+        <v>218.7</v>
+      </c>
+      <c r="D4">
+        <v>4.1794470660337089</v>
+      </c>
+      <c r="E4">
+        <v>3.2726999999999992E-2</v>
+      </c>
+      <c r="F4">
+        <v>3.3058550751322648E-4</v>
+      </c>
+      <c r="G4">
+        <v>2.3398487830376369</v>
+      </c>
+      <c r="H4">
+        <v>-1.4850938035267001</v>
+      </c>
+      <c r="I4">
+        <v>-1.4781681610696109</v>
+      </c>
       <c r="J4" s="14"/>
       <c r="K4" s="14"/>
       <c r="L4" s="14"/>
@@ -10537,14 +11617,30 @@
       <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5"/>
-      <c r="H5"/>
-      <c r="I5"/>
+      <c r="B5">
+        <v>196</v>
+      </c>
+      <c r="C5">
+        <v>480.2</v>
+      </c>
+      <c r="D5">
+        <v>2.48461935381123</v>
+      </c>
+      <c r="E5">
+        <v>2.2415000000000001E-2</v>
+      </c>
+      <c r="F5">
+        <v>2.3995948732141351E-4</v>
+      </c>
+      <c r="G5">
+        <v>2.6814221557210089</v>
+      </c>
+      <c r="H5">
+        <v>-1.649461256798189</v>
+      </c>
+      <c r="I5">
+        <v>-1.6582820305540229</v>
+      </c>
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
       <c r="L5" s="14"/>
@@ -10558,14 +11654,30 @@
       <c r="A6" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B6"/>
-      <c r="C6"/>
-      <c r="D6"/>
-      <c r="E6"/>
-      <c r="F6"/>
-      <c r="G6"/>
-      <c r="H6"/>
-      <c r="I6"/>
+      <c r="B6">
+        <v>262</v>
+      </c>
+      <c r="C6">
+        <v>862.5</v>
+      </c>
+      <c r="D6">
+        <v>4.7755162606314672</v>
+      </c>
+      <c r="E6">
+        <v>1.6105999999999999E-2</v>
+      </c>
+      <c r="F6">
+        <v>8.7866059684296963E-5</v>
+      </c>
+      <c r="G6">
+        <v>2.9357591037453119</v>
+      </c>
+      <c r="H6">
+        <v>-1.793012305243592</v>
+      </c>
+      <c r="I6">
+        <v>-1.7923955637654581</v>
+      </c>
       <c r="J6" s="14"/>
       <c r="K6" s="14"/>
       <c r="L6" s="14"/>
@@ -10579,14 +11691,30 @@
       <c r="A7" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
-      <c r="I7"/>
+      <c r="B7">
+        <v>328</v>
+      </c>
+      <c r="C7">
+        <v>1345.8</v>
+      </c>
+      <c r="D7">
+        <v>5.6819402007100033</v>
+      </c>
+      <c r="E7">
+        <v>1.2688E-2</v>
+      </c>
+      <c r="F7">
+        <v>7.8709028142336492E-5</v>
+      </c>
+      <c r="G7">
+        <v>3.1289805239666109</v>
+      </c>
+      <c r="H7">
+        <v>-1.8966068300264709</v>
+      </c>
+      <c r="I7">
+        <v>-1.894282480154553</v>
+      </c>
       <c r="J7" s="14"/>
       <c r="K7" s="14"/>
       <c r="L7" s="14"/>
@@ -10600,14 +11728,30 @@
       <c r="A8" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B8"/>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8"/>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8"/>
+      <c r="B8">
+        <v>393</v>
+      </c>
+      <c r="C8">
+        <v>1950.4</v>
+      </c>
+      <c r="D8">
+        <v>5.619806244188692</v>
+      </c>
+      <c r="E8">
+        <v>1.0531E-2</v>
+      </c>
+      <c r="F8">
+        <v>2.7424644229435522E-5</v>
+      </c>
+      <c r="G8">
+        <v>3.2901236882743068</v>
+      </c>
+      <c r="H8">
+        <v>-1.977530387232231</v>
+      </c>
+      <c r="I8">
+        <v>-1.9792543227674899</v>
+      </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15"/>
       <c r="L8" s="15"/>
@@ -10633,66 +11777,146 @@
       <c r="A9" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9"/>
+      <c r="B9">
+        <v>459</v>
+      </c>
+      <c r="C9">
+        <v>2662.6</v>
+      </c>
+      <c r="D9">
+        <v>4.9959983987187186</v>
+      </c>
+      <c r="E9">
+        <v>8.8640000000000004E-3</v>
+      </c>
+      <c r="F9">
+        <v>2.625515822335361E-5</v>
+      </c>
+      <c r="G9">
+        <v>3.4253059276703191</v>
+      </c>
+      <c r="H9">
+        <v>-2.052370252615646</v>
+      </c>
+      <c r="I9">
+        <v>-2.0505368001804869</v>
+      </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B10"/>
-      <c r="C10"/>
-      <c r="D10"/>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
-      <c r="I10"/>
+      <c r="B10">
+        <v>524</v>
+      </c>
+      <c r="C10">
+        <v>3464.1</v>
+      </c>
+      <c r="D10">
+        <v>4.1000000000000014</v>
+      </c>
+      <c r="E10">
+        <v>7.6649999999999999E-3</v>
+      </c>
+      <c r="F10">
+        <v>2.44608530786098E-5</v>
+      </c>
+      <c r="G10">
+        <v>3.5395904205339161</v>
+      </c>
+      <c r="H10">
+        <v>-2.1154878408096058</v>
+      </c>
+      <c r="I10">
+        <v>-2.1107997594094758</v>
+      </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B11"/>
-      <c r="C11"/>
-      <c r="D11"/>
-      <c r="E11"/>
-      <c r="F11"/>
-      <c r="G11"/>
-      <c r="H11"/>
-      <c r="I11"/>
+      <c r="B11">
+        <v>590</v>
+      </c>
+      <c r="C11">
+        <v>4413.3</v>
+      </c>
+      <c r="D11">
+        <v>7.7172965905598483</v>
+      </c>
+      <c r="E11">
+        <v>6.7539999999999987E-3</v>
+      </c>
+      <c r="F11">
+        <v>1.034944979750663E-5</v>
+      </c>
+      <c r="G11">
+        <v>3.644763450201828</v>
+      </c>
+      <c r="H11">
+        <v>-2.1704389437006069</v>
+      </c>
+      <c r="I11">
+        <v>-2.1662581846083468</v>
+      </c>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B12"/>
-      <c r="C12"/>
-      <c r="D12"/>
-      <c r="E12"/>
-      <c r="F12"/>
-      <c r="G12"/>
-      <c r="H12"/>
-      <c r="I12"/>
+      <c r="B12">
+        <v>656</v>
+      </c>
+      <c r="C12">
+        <v>5475.3</v>
+      </c>
+      <c r="D12">
+        <v>2.4857370916669539</v>
+      </c>
+      <c r="E12">
+        <v>6.0280000000000004E-3</v>
+      </c>
+      <c r="F12">
+        <v>4.163331998932285E-6</v>
+      </c>
+      <c r="G12">
+        <v>3.7384079198181208</v>
+      </c>
+      <c r="H12">
+        <v>-2.2198267563574059</v>
+      </c>
+      <c r="I12">
+        <v>-2.2156375248241922</v>
+      </c>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B13"/>
-      <c r="C13"/>
-      <c r="D13"/>
-      <c r="E13"/>
-      <c r="F13"/>
-      <c r="G13"/>
-      <c r="H13"/>
-      <c r="I13"/>
+      <c r="B13">
+        <v>666</v>
+      </c>
+      <c r="C13">
+        <v>8615</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>4.9199999999999999E-3</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>3.9352552817840469</v>
+      </c>
+      <c r="H13">
+        <v>-2.3080348972326399</v>
+      </c>
+      <c r="I13">
+        <v>-2.3194364239683218</v>
+      </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="27" t="s">
@@ -11705,55 +12929,319 @@
       <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
+      <c r="C3">
+        <v>53.9</v>
+      </c>
+      <c r="D3">
+        <v>1.9174636024359539</v>
+      </c>
+      <c r="E3">
+        <v>9.7462999999999994E-2</v>
+      </c>
+      <c r="F3">
+        <v>4.4250825604350771E-3</v>
+      </c>
+      <c r="G3">
+        <v>1.731588765186739</v>
+      </c>
+      <c r="H3">
+        <v>-1.011160224768868</v>
+      </c>
+      <c r="I3">
+        <v>-0.96566965972394891</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B4">
+        <v>131</v>
+      </c>
+      <c r="C4">
+        <v>218.7</v>
+      </c>
+      <c r="D4">
+        <v>4.1794470660337089</v>
+      </c>
+      <c r="E4">
+        <v>3.3418000000000003E-2</v>
+      </c>
+      <c r="F4">
+        <v>1.4100092986297011E-3</v>
+      </c>
+      <c r="G4">
+        <v>2.3398487830376369</v>
+      </c>
+      <c r="H4">
+        <v>-1.4760195453150069</v>
+      </c>
+      <c r="I4">
+        <v>-1.4890379727906491</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>196</v>
+      </c>
+      <c r="C5">
+        <v>480.2</v>
+      </c>
+      <c r="D5">
+        <v>2.48461935381123</v>
+      </c>
+      <c r="E5">
+        <v>1.7444000000000001E-2</v>
+      </c>
+      <c r="F5">
+        <v>6.2539445330305106E-4</v>
+      </c>
+      <c r="G5">
+        <v>2.6814221557210089</v>
+      </c>
+      <c r="H5">
+        <v>-1.7583539219986111</v>
+      </c>
+      <c r="I5">
+        <v>-1.782939716458471</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>262</v>
+      </c>
+      <c r="C6">
+        <v>862.5</v>
+      </c>
+      <c r="D6">
+        <v>4.7755162606314672</v>
+      </c>
+      <c r="E6">
+        <v>1.0961E-2</v>
+      </c>
+      <c r="F6">
+        <v>5.1824586614634732E-4</v>
+      </c>
+      <c r="G6">
+        <v>2.9357591037453119</v>
+      </c>
+      <c r="H6">
+        <v>-1.960149822250336</v>
+      </c>
+      <c r="I6">
+        <v>-2.0017801720720469</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B7">
+        <v>328</v>
+      </c>
+      <c r="C7">
+        <v>1345.8</v>
+      </c>
+      <c r="D7">
+        <v>5.6819402007100033</v>
+      </c>
+      <c r="E7">
+        <v>6.6640000000000007E-3</v>
+      </c>
+      <c r="F7">
+        <v>2.905902040101604E-4</v>
+      </c>
+      <c r="G7">
+        <v>3.1289805239666109</v>
+      </c>
+      <c r="H7">
+        <v>-2.1762650116012692</v>
+      </c>
+      <c r="I7">
+        <v>-2.168034678009938</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B8">
+        <v>393</v>
+      </c>
+      <c r="C8">
+        <v>1950.4</v>
+      </c>
+      <c r="D8">
+        <v>5.619806244188692</v>
+      </c>
+      <c r="E8">
+        <v>5.1879999999999999E-3</v>
+      </c>
+      <c r="F8">
+        <v>2.0104615279968821E-4</v>
+      </c>
+      <c r="G8">
+        <v>3.2901236882743068</v>
+      </c>
+      <c r="H8">
+        <v>-2.2850000325879569</v>
+      </c>
+      <c r="I8">
+        <v>-2.306687924304061</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B9">
+        <v>459</v>
+      </c>
+      <c r="C9">
+        <v>2662.6</v>
+      </c>
+      <c r="D9">
+        <v>4.9959983987187186</v>
+      </c>
+      <c r="E9">
+        <v>3.7309999999999999E-3</v>
+      </c>
+      <c r="F9">
+        <v>6.3112773843511448E-5</v>
+      </c>
+      <c r="G9">
+        <v>3.4253059276703191</v>
+      </c>
+      <c r="H9">
+        <v>-2.4281747509591711</v>
+      </c>
+      <c r="I9">
+        <v>-2.4230034777071001</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B10">
+        <v>524</v>
+      </c>
+      <c r="C10">
+        <v>3464.1</v>
+      </c>
+      <c r="D10">
+        <v>4.1000000000000014</v>
+      </c>
+      <c r="E10">
+        <v>3.0590000000000001E-3</v>
+      </c>
+      <c r="F10">
+        <v>2.172811798364303E-5</v>
+      </c>
+      <c r="G10">
+        <v>3.5395904205339161</v>
+      </c>
+      <c r="H10">
+        <v>-2.5144205230153212</v>
+      </c>
+      <c r="I10">
+        <v>-2.521337874978574</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B11">
+        <v>590</v>
+      </c>
+      <c r="C11">
+        <v>4413.3</v>
+      </c>
+      <c r="D11">
+        <v>7.7172965905598483</v>
+      </c>
+      <c r="E11">
+        <v>2.4269999999999999E-3</v>
+      </c>
+      <c r="F11">
+        <v>2.24127939653523E-5</v>
+      </c>
+      <c r="G11">
+        <v>3.644763450201828</v>
+      </c>
+      <c r="H11">
+        <v>-2.6149302236680652</v>
+      </c>
+      <c r="I11">
+        <v>-2.6118324488483009</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B12">
+        <v>656</v>
+      </c>
+      <c r="C12">
+        <v>5475.3</v>
+      </c>
+      <c r="D12">
+        <v>2.4857370916669539</v>
+      </c>
+      <c r="E12">
+        <v>2.042E-3</v>
+      </c>
+      <c r="F12">
+        <v>6.9358969619413063E-5</v>
+      </c>
+      <c r="G12">
+        <v>3.7384079198181208</v>
+      </c>
+      <c r="H12">
+        <v>-2.6899442622491092</v>
+      </c>
+      <c r="I12">
+        <v>-2.6924074441673569</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>4</v>
+      </c>
+      <c r="B13">
+        <v>666</v>
+      </c>
+      <c r="C13">
+        <v>8615</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>1.23E-3</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>3.9352552817840469</v>
+      </c>
+      <c r="H13">
+        <v>-2.9100948885606019</v>
+      </c>
+      <c r="I13">
+        <v>-2.8617818379138669</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -12767,55 +14255,319 @@
       <c r="A3" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
+      <c r="C3">
+        <v>53.9</v>
+      </c>
+      <c r="D3">
+        <v>1.9174636024359539</v>
+      </c>
+      <c r="E3">
+        <v>0.22412399999999999</v>
+      </c>
+      <c r="F3">
+        <v>6.2449907392512069E-3</v>
+      </c>
+      <c r="G3">
+        <v>1.731588765186739</v>
+      </c>
+      <c r="H3">
+        <v>-0.64951163516741062</v>
+      </c>
+      <c r="I3">
+        <v>-0.63677377983195127</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B4">
+        <v>131</v>
+      </c>
+      <c r="C4">
+        <v>218.7</v>
+      </c>
+      <c r="D4">
+        <v>4.1794470660337089</v>
+      </c>
+      <c r="E4">
+        <v>0.126966</v>
+      </c>
+      <c r="F4">
+        <v>1.886533682003409E-3</v>
+      </c>
+      <c r="G4">
+        <v>2.3398487830376369</v>
+      </c>
+      <c r="H4">
+        <v>-0.89631256242428237</v>
+      </c>
+      <c r="I4">
+        <v>-0.90505447920028792</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>196</v>
+      </c>
+      <c r="C5">
+        <v>480.2</v>
+      </c>
+      <c r="D5">
+        <v>2.48461935381123</v>
+      </c>
+      <c r="E5">
+        <v>8.7507000000000001E-2</v>
+      </c>
+      <c r="F5">
+        <v>9.8419515905693667E-4</v>
+      </c>
+      <c r="G5">
+        <v>2.6814221557210089</v>
+      </c>
+      <c r="H5">
+        <v>-1.0579572048088031</v>
+      </c>
+      <c r="I5">
+        <v>-1.055709693450388</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B6">
+        <v>262</v>
+      </c>
+      <c r="C6">
+        <v>862.5</v>
+      </c>
+      <c r="D6">
+        <v>4.7755162606314672</v>
+      </c>
+      <c r="E6">
+        <v>6.9010000000000002E-2</v>
+      </c>
+      <c r="F6">
+        <v>2.1445538256502451E-4</v>
+      </c>
+      <c r="G6">
+        <v>2.9357591037453119</v>
+      </c>
+      <c r="H6">
+        <v>-1.1610879725940011</v>
+      </c>
+      <c r="I6">
+        <v>-1.1678881899628679</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B7">
+        <v>328</v>
+      </c>
+      <c r="C7">
+        <v>1345.8</v>
+      </c>
+      <c r="D7">
+        <v>5.6819402007100033</v>
+      </c>
+      <c r="E7">
+        <v>5.6743000000000009E-2</v>
+      </c>
+      <c r="F7">
+        <v>4.1406668813395568E-4</v>
+      </c>
+      <c r="G7">
+        <v>3.1289805239666109</v>
+      </c>
+      <c r="H7">
+        <v>-1.246087706802355</v>
+      </c>
+      <c r="I7">
+        <v>-1.2531109174619821</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B8">
+        <v>393</v>
+      </c>
+      <c r="C8">
+        <v>1950.4</v>
+      </c>
+      <c r="D8">
+        <v>5.619806244188692</v>
+      </c>
+      <c r="E8">
+        <v>4.7560000000000012E-2</v>
+      </c>
+      <c r="F8">
+        <v>1.6349651712226521E-4</v>
+      </c>
+      <c r="G8">
+        <v>3.2901236882743068</v>
+      </c>
+      <c r="H8">
+        <v>-1.322758154053346</v>
+      </c>
+      <c r="I8">
+        <v>-1.3241851284082169</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B9">
+        <v>459</v>
+      </c>
+      <c r="C9">
+        <v>2662.6</v>
+      </c>
+      <c r="D9">
+        <v>4.9959983987187186</v>
+      </c>
+      <c r="E9">
+        <v>4.1593999999999999E-2</v>
+      </c>
+      <c r="F9">
+        <v>8.9668525383461247E-5</v>
+      </c>
+      <c r="G9">
+        <v>3.4253059276703191</v>
+      </c>
+      <c r="H9">
+        <v>-1.380969312518098</v>
+      </c>
+      <c r="I9">
+        <v>-1.383808948259927</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B10">
+        <v>524</v>
+      </c>
+      <c r="C10">
+        <v>3464.1</v>
+      </c>
+      <c r="D10">
+        <v>4.1000000000000014</v>
+      </c>
+      <c r="E10">
+        <v>3.7127E-2</v>
+      </c>
+      <c r="F10">
+        <v>9.4997660789913915E-5</v>
+      </c>
+      <c r="G10">
+        <v>3.5395904205339161</v>
+      </c>
+      <c r="H10">
+        <v>-1.430310141969187</v>
+      </c>
+      <c r="I10">
+        <v>-1.434215555257919</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B11">
+        <v>590</v>
+      </c>
+      <c r="C11">
+        <v>4413.3</v>
+      </c>
+      <c r="D11">
+        <v>7.7172965905598483</v>
+      </c>
+      <c r="E11">
+        <v>3.3199999999999993E-2</v>
+      </c>
+      <c r="F11">
+        <v>3.0073982849706361E-5</v>
+      </c>
+      <c r="G11">
+        <v>3.644763450201828</v>
+      </c>
+      <c r="H11">
+        <v>-1.478861916295964</v>
+      </c>
+      <c r="I11">
+        <v>-1.4806034372918011</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>4</v>
       </c>
+      <c r="B12">
+        <v>656</v>
+      </c>
+      <c r="C12">
+        <v>5475.3</v>
+      </c>
+      <c r="D12">
+        <v>2.4857370916669539</v>
+      </c>
+      <c r="E12">
+        <v>3.0089000000000001E-2</v>
+      </c>
+      <c r="F12">
+        <v>1.3453624047073539E-5</v>
+      </c>
+      <c r="G12">
+        <v>3.7384079198181208</v>
+      </c>
+      <c r="H12">
+        <v>-1.5215922456829389</v>
+      </c>
+      <c r="I12">
+        <v>-1.5219065035189721</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="27" t="s">
         <v>4</v>
+      </c>
+      <c r="B13">
+        <v>666</v>
+      </c>
+      <c r="C13">
+        <v>8615</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>2.3630000000000009E-2</v>
+      </c>
+      <c r="F13">
+        <v>1.1564823173178709E-18</v>
+      </c>
+      <c r="G13">
+        <v>3.9352552817840469</v>
+      </c>
+      <c r="H13">
+        <v>-1.6265362783676309</v>
+      </c>
+      <c r="I13">
+        <v>-1.6087284980397041</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>